<commit_message>
Fix Excel state store: add missing deferred_until column to pipeline_state sheet
Column was in _STATE_COLS but absent from the initialized header row — would have caused
silent key errors on first DEFER command. Now matches code exactly.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/invoice_pipeline_state.xlsx
+++ b/data/invoice_pipeline_state.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,10 +510,15 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>deferred_until</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>

</xml_diff>

<commit_message>
fix: reset 50 orders from details_missing -> invoice_needed (FTF API was empty, now set)
</commit_message>
<xml_diff>
--- a/data/invoice_pipeline_state.xlsx
+++ b/data/invoice_pipeline_state.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="pipeline_state" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="learnings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="pending_confirmations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="poll_state" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_state" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="learnings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pending_confirmations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="poll_state" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -534,7 +534,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:10.795898+00:00</t>
+          <t>2026-06-02T13:04:37.168006</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:12.955138+00:00</t>
+          <t>2026-06-02T13:04:37.168071</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:15.026819+00:00</t>
+          <t>2026-06-02T13:04:37.168103</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:17.019754+00:00</t>
+          <t>2026-06-02T13:04:37.168127</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:18.819123+00:00</t>
+          <t>2026-06-02T13:04:37.168151</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:20.744754+00:00</t>
+          <t>2026-06-02T13:04:37.168175</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:22.645338+00:00</t>
+          <t>2026-06-02T13:04:37.168199</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:24.715250+00:00</t>
+          <t>2026-06-02T13:04:37.168223</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:26.582321+00:00</t>
+          <t>2026-06-02T13:04:37.168254</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:28.425258+00:00</t>
+          <t>2026-06-02T13:04:37.168277</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:30.421924+00:00</t>
+          <t>2026-06-02T13:04:37.168300</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:32.468006+00:00</t>
+          <t>2026-06-02T13:04:37.168325</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:34.316542+00:00</t>
+          <t>2026-06-02T13:04:37.168349</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:36.248610+00:00</t>
+          <t>2026-06-02T13:04:37.168372</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:38.620134+00:00</t>
+          <t>2026-06-02T13:04:37.168396</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:40.514627+00:00</t>
+          <t>2026-06-02T13:04:37.168419</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:42.296615+00:00</t>
+          <t>2026-06-02T13:04:37.168442</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:44.345161+00:00</t>
+          <t>2026-06-02T13:04:37.168479</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:46.184244+00:00</t>
+          <t>2026-06-02T13:04:37.168502</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:48.143958+00:00</t>
+          <t>2026-06-02T13:04:37.168525</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:50.131578+00:00</t>
+          <t>2026-06-02T13:04:37.168548</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:51.888477+00:00</t>
+          <t>2026-06-02T13:04:37.168571</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:53.710262+00:00</t>
+          <t>2026-06-02T13:04:37.168593</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:55.682901+00:00</t>
+          <t>2026-06-02T13:04:37.168617</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:57.678533+00:00</t>
+          <t>2026-06-02T13:04:37.168638</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>2026-06-02T12:17:59.534323+00:00</t>
+          <t>2026-06-02T13:04:37.168660</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:01.503498+00:00</t>
+          <t>2026-06-02T13:04:37.168688</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:03.358452+00:00</t>
+          <t>2026-06-02T13:04:37.168710</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:05.144257+00:00</t>
+          <t>2026-06-02T13:04:37.168733</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:07.049188+00:00</t>
+          <t>2026-06-02T13:04:37.168757</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1939,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:08.893955+00:00</t>
+          <t>2026-06-02T13:04:37.168779</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:10.883374+00:00</t>
+          <t>2026-06-02T13:04:37.168802</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:12.724362+00:00</t>
+          <t>2026-06-02T13:04:37.168825</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:14.638582+00:00</t>
+          <t>2026-06-02T13:04:37.168848</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:16.509012+00:00</t>
+          <t>2026-06-02T13:04:37.168870</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2174,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:19.189772+00:00</t>
+          <t>2026-06-02T13:04:37.168893</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:21.216665+00:00</t>
+          <t>2026-06-02T13:04:37.168915</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:23.012989+00:00</t>
+          <t>2026-06-02T13:04:37.168937</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:24.964370+00:00</t>
+          <t>2026-06-02T13:04:37.168961</t>
         </is>
       </c>
     </row>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:26.922983+00:00</t>
+          <t>2026-06-02T13:04:37.168983</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:29.256357+00:00</t>
+          <t>2026-06-02T13:04:37.169006</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:31.172123+00:00</t>
+          <t>2026-06-02T13:04:37.169031</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:33.122199+00:00</t>
+          <t>2026-06-02T13:04:37.169053</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:34.975751+00:00</t>
+          <t>2026-06-02T13:04:37.169076</t>
         </is>
       </c>
     </row>
@@ -2597,7 +2597,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:36.798698+00:00</t>
+          <t>2026-06-02T13:04:37.169100</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:38.576208+00:00</t>
+          <t>2026-06-02T13:04:37.169123</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:40.600270+00:00</t>
+          <t>2026-06-02T13:04:37.169146</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:42.499578+00:00</t>
+          <t>2026-06-02T13:04:37.169170</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:45.649012+00:00</t>
+          <t>2026-06-02T13:04:37.169193</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>details_missing</t>
+          <t>invoice_needed</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2026-06-02T12:18:47.452843+00:00</t>
+          <t>2026-06-02T13:04:37.169215</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: advance order 1000273343 to invoice_approved + clean up Teams card
- Manually set order 1000273343 status=invoice_approved (approved_by=Prateek)
  Teams reply at 12:53 AM IST was not picked up by poller; advancing directly
  so A5/A6 can complete the pipeline on next cycle.

- Remove synonym hints from approval card display in A3.
  AI still understands all synonyms internally — just not shown to users.
</commit_message>
<xml_diff>
--- a/data/invoice_pipeline_state.xlsx
+++ b/data/invoice_pipeline_state.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="pipeline_state" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="learnings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="pending_confirmations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="poll_state" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_state" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="learnings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pending_confirmations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="poll_state" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>invoice_draft_posted</t>
+          <t>invoice_approved</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -11549,6 +11549,11 @@
           <t>2026-06-02T19:20:20.753326+00:00</t>
         </is>
       </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>Prateek</t>
+        </is>
+      </c>
       <c r="R174" t="n">
         <v>475</v>
       </c>
@@ -11559,7 +11564,7 @@
       </c>
       <c r="U174" t="inlineStr">
         <is>
-          <t>2026-06-02T19:20:20.810846+00:00</t>
+          <t>2026-06-02T19:42:31.451877+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: set 1000273343 to invoice_finalized — EMAIL_OVERRIDE_ALL check
</commit_message>
<xml_diff>
--- a/data/invoice_pipeline_state.xlsx
+++ b/data/invoice_pipeline_state.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="pipeline_state" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="learnings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="pending_confirmations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="poll_state" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_state" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="learnings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pending_confirmations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="poll_state" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>invoice_approved</t>
+          <t>invoice_finalized</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -11539,6 +11539,11 @@
       <c r="J174" t="n">
         <v>0</v>
       </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>TEST-OVERRIDE-CHECK</t>
+        </is>
+      </c>
       <c r="L174" t="inlineStr">
         <is>
           <t>2026-06-02T18:01:01.624011+00:00</t>
@@ -11564,7 +11569,7 @@
       </c>
       <c r="U174" t="inlineStr">
         <is>
-          <t>2026-06-02T19:42:31.451877+00:00</t>
+          <t>2026-06-02T20:05:31.763216+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(intake): DB restored — seed sheet with recent orders, watermark to recent floor
MySQL/RDS reachable again. Set intake watermark to ng_id 52360151 (last ~2 days,
28 eligible invoice-needed orders) so the sheet fills with current work and excludes
the ~344 stale older orders. Ran A1->A2->A3 once: 10 queued, 9 data-collected,
9 posted to the Approvals sheet (8 priced drafts $300-$725 + 1 condo auto-reject).
Committing state so CI dedups against these and keeps draining 10/run.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/invoice_pipeline_state.xlsx
+++ b/data/invoice_pipeline_state.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,6 +528,700 @@
       <c r="V1" t="inlineStr">
         <is>
           <t>pay_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1000285900</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>marcosjunkemail@yahoo.com</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4509 NW 53RD ST, GAINESVILLE, FL 32606</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>{"total_amount": 649.0, "services": [{"name": "Boundary Survey (Base Rate)", "description": "Standard residential boundary survey for individual client Marco at 4509 NW 53rd St, Gainesville, FL. Default individual client base rate applied.", "amount": 475.0}, {"name": "Lot Size Upcharge (0.31\u20130.50 ac)", "description": "Aerial analysis estimates lot at approximately 0.45 acres, placing it in the 0.31\u20130.50 ac tier. Upcharge applied accordingly.", "amount": 62.0}, {"name": "Heavy Vegetation Upcharge", "description": "Aerial imagery confirms dense tree canopy heavily obscuring lot boundaries and ground features. Site notes indicate tree clearing may be required for accurate boundary staking. Heavy vegetation upcharge is warranted.", "amount": 112.0}], "pricing_reasoning": "No specific survey service was identified in the order, so a standard boundary survey is assumed as the most likely service for a residential individual client quote request with a MARCO certification noted. The lot is estimated at ~0.45 acres via aerial analysis (no county appraiser data available), triggering the 0.31\u20130.50 ac size upcharge. Heavy vegetation is clearly supported by aerial imagery showing dense canopy, curved shared access, and difficult-to-determine lot boundaries, justifying the vegetation upcharge. No pool, waterfront, Monroe County, FEMA flood zone, or metes-and-bounds complexity was identified.", "confidence": "LOW", "escalate_flag": true, "escalate_reason": "The specific survey service requested has not been identified by the client. The county appraiser site was unreachable, so lot size, legal description, and FEMA flood zone could not be confirmed \u2014 all pricing relies on aerial estimation only. Management should confirm: (1) intended service type, (2) whether an Elevation Certificate is needed given unknown FEMA zone, (3) whether a topographic survey is required given apparent elevation changes noted in aerial analysis, and (4) verify lot size via county records before finalizing the quote.", "flags": ["No service type specified \u2014 boundary survey assumed as default for quote purposes.", "County appraiser site unreachable \u2014 lot size (~0.45 ac), legal description, and FEMA flood zone are unverified. All aerial-derived estimates carry LOW confidence.", "FEMA flood zone unknown \u2014 if property falls in a flood zone, an Elevation Certificate line item may need to be added.", "Aerial imagery suggests possible shared or curved private road serving multiple parcels \u2014 easement or access complexity may require additional field time.", "Elevation changes noted in aerial analysis \u2014 if topographic survey is requested, pricing would be $825.00 for a 0.31\u20130.50 ac lot per topo schedule, replacing the boundary survey line items."]}</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202606242245369831, "created_at": "2026-06-24T22:45:37", "customer_email": "marcosjunkemail@yahoo.com", "customer_id": 202606242245369942, "customer_name": "Marco", "customer_type": "individual", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": null, "invoiced": false, "order_id": 1000285900, "paid": false, "property_address": "4509 NW 53RD ST", "property_city": "GAINESVILLE", "property_county": "Alachua County", "property_lat": "29.6963418", "property_lng": "-82.39950669999999", "property_state": "FLORIDA", "property_zip": "32606", "service_type": "Quote", "special_pricing": false, "status": "Quote", "status_code": 12, "updated_at": "2026-06-24T22:45:42"}, "ftf_customer": {"data": {"company_id": 202606242245369831, "company_name": "Marco", "created_at": null, "custom_rate": null, "customer_id": 202606242245369942, "customer_type": "individual", "email": "marcosjunkemail@yahoo.com", "first_name": "Marco", "last_name": " ", "phone": "954-235-5853", "pricing_type": 0, "special_pricing": false}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": null, "source_url": "https://qpublic.schneidercorp.com/Application.aspx?AppID=1081&amp;LayerID=26490&amp;PageTypeID=4&amp;PageID=10770&amp;Q=168079894&amp;KeyValue=", "confidence": "LOW", "error": "Appraiser site unreachable (possible broken URL): https://qpublic.schneidercorp.com/Application.aspx?AppID=1081&amp;LayerID=26490&amp;PageTypeID=4&amp;PageID=10770&amp;Q=168079894&amp;KeyValue="}, "aerial_analysis": {"lot_shape": "irregular", "estimated_lot_size": "~0.45 acres", "main_structure_footprint_sqft": 2800, "visible_structures": ["main house"], "driveway_count": 1, "pool_visible": false, "apparent_encroachments": null, "access_type": "street", "site_notes": "Property is heavily wooded with dense tree canopy obscuring significant portions of the lot boundaries and ground features. Curved private road or shared drive appears to serve multiple parcels in this subdivision. Lot boundaries are difficult to determine precisely due to vegetation coverage. Surrounding area contains multiple similarly wooded residential lots. Elevation changes may be present given the natural tree density and apparent topographic variation. Tree clearing may be required for accurate boundary staking.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Marco", "confidence": "HIGH"}, "client_email": {"value": "marcosjunkemail@yahoo.com", "confidence": "HIGH"}, "property_address": {"value": "4509 NW 53RD ST, GAINESVILLE, FL 32606", "confidence": "HIGH"}, "property_county": {"value": "Alachua County", "confidence": "HIGH"}, "services_requested": {"value": ["Quote"], "confidence": "LOW", "notes": "Service type is listed only as 'Quote' \u2014 no specific survey type (boundary, topographic, elevation cert, etc.) has been identified yet. Needs clarification."}, "special_requirements": {"value": null, "confidence": "LOW"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features available \u2014 county appraiser site unreachable and no emails or aerial data provided."}, "client_tier": {"value": "residential", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Specific survey type or service requested is unknown \u2014 only 'Quote' status present", "Lot size not available \u2014 county appraiser site unreachable", "Legal description not available \u2014 county appraiser site unreachable", "Structure square footage unknown", "Property features (pool, shed, fences, etc.) unknown", "No special requirements or notes from client", "No matching emails found to clarify scope", "Last name for client is blank \u2014 only first name 'Marco' on file"], "summary": "Individual client Marco submitted a quote request for a property at 4509 NW 53rd St, Gainesville, FL (Alachua County), but no specific survey service has been identified and property details are unavailable due to the county appraiser site being unreachable."}}</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1000285900</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:49.455048+00:00</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-25 05:34 EDT</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>649</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:34:07.704511+00:00</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:03.549944+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1000285895</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Land Survey and Elevation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>amanda@encoretitlegroup.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Amanda Burnett (Encore Title Group LLC)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>816 Columbus Ave, Lehigh Acres, FL 33972</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>{"total_amount": 637.0, "services": [{"name": "Boundary Survey", "description": "Standard boundary survey at negotiated OLD_TITLE client rate for Encore Title Group LLC. Base rate per management-agreed pricing.", "amount": 300.0}, {"name": "Lot Size Complexity Upcharge (0.31\u20130.50 ac)", "description": "Database lot size is 0.50 acres, which falls in the 0.31\u20130.50 ac complexity tier. Aerial analysis estimates ~0.8 ac, but the legal description and DB value of 0.50 ac are the authoritative reference for pricing; upcharge applied at the lower confirmed tier. Active construction, disturbed markers, and urban corner lot add to field complexity supporting this charge.", "amount": 62.0}, {"name": "Elevation Certificate (EC)", "description": "FEMA Flood Zone AE elevation certificate. Standard EC rate; VE coastal premium does not apply as zone is AE, not VE.", "amount": 275.0}], "pricing_reasoning": "This is a combined boundary survey and elevation certificate order in Lee County, Flood Zone AE. The negotiated base survey rate of $300.00 for Encore Title Group LLC is applied per management agreement, with a $62.00 lot size upcharge for the 0.31\u20130.50 ac tier based on the authoritative DB lot size of 0.50 acres. The EC is priced at the fixed $275.00 rate; no VE surcharge applies. The aerial analysis flagged significant construction activity, disturbed markers, and a complex urban corner lot, which are captured by the lot size complexity upcharge \u2014 no additional metes-and-bounds or other upcharges are warranted given the straightforward platted legal description.", "confidence": "MEDIUM", "escalate_flag": false, "escalate_reason": null, "flags": ["AERIAL_LOT_SIZE_DISCREPANCY: Aerial analysis estimates ~0.8 acres while DB records 0.50 acres. Platted legal description and DB value used as authoritative basis; if field crew confirms lot is materially larger, upcharge tier should be revisited (0.51\u20131.00 ac = +$137.00 replacing the $62.00 upcharge, net +$75.00 adjustment).", "AERIAL_CONFIDENCE_LOW: Google satellite analysis returned LOW confidence due to active construction, crane, and staging equipment obscuring lot boundaries. Field crew should verify survey monuments and right-of-way limits carefully.", "CONSTRUCTION_ENCROACHMENT: Active construction crane and staging equipment may extend into public right-of-way and adjacent parcels. Crew should document and notify client if encroachments are confirmed.", "NEW_CLIENT_ZERO_ORDERS: Encore Title Group LLC shows 0 prior orders with NexGen despite being classified OLD_TITLE. Negotiated rate applied as instructed; no further action required but noted for records."]}</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202402221922288632, "created_at": "2026-06-24T20:10:27", "customer_email": "amanda@encoretitlegroup.com", "customer_id": 202402221922538535, "customer_name": "AMANDA  BURNETT", "customer_type": "b2b", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12071C0339F\nZONE: AE\nELEV: 23 FT\nEFF: 08/28/2008", "invoiced": false, "order_id": 1000285895, "paid": false, "property_address": "816 COLUMBUS AVE", "property_city": "LEHIGH ACRES", "property_county": "LEE COUNTY", "property_lat": "26.6316027", "property_lng": "-81.5871999", "property_state": "FL", "property_zip": "33972", "service_type": "Land Survey and Elevation", "special_pricing": true, "status": "In-Field", "status_code": 3, "updated_at": "2026-06-24T21:40:39"}, "ftf_customer": {"data": {"company_id": 202402221922288632, "company_name": "Encore Title Group LLC", "created_at": null, "custom_rate": 300.0, "customer_id": 202402221922538535, "customer_type": "b2b", "email": "amanda@encoretitlegroup.com", "first_name": "AMANDA ", "last_name": "BURNETT", "phone": "2399943447", "pricing_type": 0, "special_pricing": true}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "No property data was returned in the page text. The page only shows the Lee County Property Appraiser website navigation and general content. The search for 816 COLUMBUS AVE did not return specific parcel details in the provided text.", "source_url": "https://www.leepa.org/?address=816%20COLUMBUS%20AVE", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "irregular", "estimated_lot_size": "~0.8 acres", "main_structure_footprint_sqft": 28000, "visible_structures": ["main multi-story residential building (under construction/renovation)", "adjacent large institutional building", "surface parking lot", "landscaped courtyard/park area", "construction crane and staging area"], "driveway_count": 2, "pool_visible": false, "apparent_encroachments": "Active construction activity with crane and equipment potentially extending beyond property boundaries into adjacent sidewalk and street areas; construction staging may overlap public right-of-way", "access_type": "street", "site_notes": "Site appears to be undergoing significant construction or major renovation. Large surface parking lot visible adjacent to structure. Corner lot at busy urban intersection with crosswalks and traffic signals visible. Proximity to large institutional/academic building to the northeast. Courtyard/green space with circular feature (fountain or plaza) visible to the south. Urban density requires careful boundary delineation. Construction activity may have disturbed original survey markers. Multiple curb cuts and pedestrian infrastructure nearby. Columbus Avenue intersection likely creates complex right-of-way considerations.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Amanda Burnett (Encore Title Group LLC)", "confidence": "HIGH"}, "client_email": {"value": "amanda@encoretitlegroup.com", "confidence": "HIGH"}, "property_address": {"value": "816 Columbus Ave, Lehigh Acres, FL 33972", "confidence": "HIGH"}, "property_county": {"value": "Lee County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey", "Elevation Certificate"], "confidence": "HIGH", "notes": "Service type listed as 'Land Survey and Elevation'; elevation_cert flag is false but service type explicitly includes elevation \u2014 may be a data entry inconsistency requiring review"}, "special_requirements": {"value": "Special pricing applied; Flood Zone AE, FEMA panel 12071C0339F, base elevation 23 ft, effective 08/28/2008", "confidence": "HIGH"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features available; no emails or attachments found to supplement"}, "client_tier": {"value": "b2b", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Lot size not provided", "Legal description not provided", "Structure square footage unknown", "Property features unknown (pool, shed, fences, etc.)", "Conflict between service_type ('Land Survey and Elevation') and elevation_cert flag (false) \u2014 needs clarification", "No supporting emails or attachments found", "Fieldwork date not yet scheduled", "Invoice not yet generated"], "summary": "B2B order from Encore Title Group LLC for a combined land survey and elevation certificate at 816 Columbus Ave, Lehigh Acres, FL (Flood Zone AE), currently in-field status with special pricing applied and no invoice issued yet."}}</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1000285895</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:26:27.559898+00:00</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-25 05:34 EDT</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>637</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:34:36.095287+00:00</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:03.685134+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1000285885</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>bbeckman@libertypools.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Brayan Beckman</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>417 Seneca Ln, Boca Raton, FL 33487</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>{"total_amount": 537.0, "services": [{"name": "Land Survey Only", "description": "Boundary survey for residential lot at 417 Seneca Ln, Boca Raton, FL 33487. Standard rectangular lot (~0.17\u20130.20 ac) in a well-defined subdivision grid. Individual client base rate applied.", "amount": 475.0}, {"name": "Pool Complexity Upcharge", "description": "Pool is clearly visible in aerial imagery in the rear yard. Pool structures require additional staking and location work during boundary survey fieldwork.", "amount": 62.0}], "pricing_reasoning": "Base rate of $475.00 is applied per the default individual client rate for NexGen. The aerial image confirms a pool in the rear yard, supporting the $62.00 pool upcharge. Lot size is 0.17 ac per database (aerial estimate ~0.20 ac), both well under the 0.31 ac threshold for a lot-size upcharge. FEMA Zone X carries no flood zone premium, no EC was requested, the lot is not waterfront, legal description shows no metes-and-bounds complexity, and the county is Palm Beach (no Monroe surcharge). No other complexity factors are supported by the available data.", "confidence": "MEDIUM", "escalate_flag": false, "escalate_reason": null, "flags": ["DUPLICATE ORDER WARNING: Order 1000285885 appears to be a duplicate of Order 1000271474 (417 Seneca Ln, Palm Beach County, Land Survey Only, same folio 06434632390180170). Human review required before scheduling or invoicing.", "DUPLICATE ORDER WARNING: Order 1000285885 also matches Order 1000283586 (417 Seneca Ln, Palm Beach County, Land Survey Only, same folio 06434632390180170). This property has now been ordered three times \u2014 confirm with client whether prior orders were completed, cancelled, or are still active before proceeding.", "Aerial analysis confidence is LOW \u2014 lot size estimate (~0.20 ac) is slightly above the database value (0.17 ac) but both fall below the 0.31 ac upcharge threshold, so no lot-size upcharge is triggered. If legal description or survey plat reveals additional complexity (e.g., metes and bounds, easements), pricing should be revisited.", "No legal description text was provided in the order. If legal description contains metes and bounds language, a $100.00 upcharge should be added."]}</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202605111938439244, "created_at": "2026-06-24T18:31:18", "customer_email": "bbeckman@libertypools.com", "customer_id": 202605111938439347, "customer_name": "Brayan Beckman", "customer_type": "individual", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12099C0987G\nZONE:X\nEFF: 12/20/2024", "invoiced": false, "order_id": 1000285885, "paid": false, "property_address": "417 SENECA LN", "property_city": "BOCA RATON", "property_county": "Palm Beach County", "property_lat": "26.419568", "property_lng": "-80.0866285", "property_state": "FLORIDA", "property_zip": "33487", "service_type": "Land Survey Only", "special_pricing": false, "status": "Quote", "status_code": 12, "updated_at": "2026-06-24T18:54:25"}, "ftf_customer": {"data": {"company_id": 202605111938439244, "company_name": "Brayan Beckman", "created_at": null, "custom_rate": null, "customer_id": 202605111938439347, "customer_type": "individual", "email": "bbeckman@libertypools.com", "first_name": "Brayan Beckman", "last_name": " ", "phone": "(561)484-4922", "pricing_type": 0, "special_pricing": false}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "No property-specific data was returned in the page text. The page appears to have loaded the Palm Beach County Property Appraiser homepage rather than the individual property detail page for 417 SENECA LN. A direct lookup on https://pbcpao.gov may be required to retrieve parcel data.", "source_url": "https://pbcpao.gov/?address=417%20SENECA%20LN", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "rectangular", "estimated_lot_size": "~0.20 acres", "main_structure_footprint_sqft": 2200, "visible_structures": ["main house", "pool"], "driveway_count": 1, "pool_visible": true, "apparent_encroachments": null, "access_type": "street", "site_notes": "Residential subdivision with uniform lot sizes and consistent setbacks. Palm trees along street frontage may require consideration for root encroachment near boundary lines. Pool appears to be in rear yard with adequate setback. Street grid is well-defined. Lot appears to conform to neighboring parcels in size and orientation.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Brayan Beckman", "confidence": "HIGH"}, "client_email": {"value": "bbeckman@libertypools.com", "confidence": "HIGH"}, "property_address": {"value": "417 Seneca Ln, Boca Raton, FL 33487", "confidence": "HIGH"}, "property_county": {"value": "Palm Beach County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated as 'Land Survey Only'; no elevation certificate requested."}, "special_requirements": {"value": null, "confidence": "LOW"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features available; no emails, attachments, or aerial data provided."}, "client_tier": {"value": "residential", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Lot size unknown \u2014 needed for accurate quote", "Legal description not provided", "Structure square footage unknown", "Property features (pool, shed, fence, driveway, etc.) not documented", "Special requirements or access notes not provided", "No fieldwork or delivery date scheduled yet", "Order is still in 'Quote' status \u2014 not yet invoiced or paid", "No matching emails found to supplement order details"], "summary": "Individual residential client Brayan Beckman is requesting a Land Survey Only at 417 Seneca Ln, Boca Raton, FL 33487 (Palm Beach County), currently in Quote status with no scheduling, pricing, or property detail information on file."}}</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1000285885</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:27:01.667431+00:00</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-25 05:34 EDT</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>537</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:35:03.200180+00:00</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:03.801057+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1000285867</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nfroio@networkcraze.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Nick Froio</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>261 Bocilla Dr, Placida, FL 33946</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>{"total_amount": 624.0, "services": [{"name": "Land Survey (Boundary)", "description": "Base residential boundary survey rate for individual client in Charlotte County. Rectangular lot ~0.20-0.24 acres, single-family home with pool, waterfront/dock.", "amount": 475.0}, {"name": "Pool Complexity Upcharge", "description": "Pool is confirmed visible in aerial imagery; pool structures must be located and shown on survey.", "amount": 62.0}, {"name": "Waterfront Canal Complexity Upcharge", "description": "Property is waterfront on western side with dock/pier extending into canal or bay. Waterfront boundary (mean high water line or platted line) and dock/pier location add field and drafting complexity.", "amount": 87.0}], "pricing_reasoning": "Base rate of $475.00 applies as a new individual residential client with no negotiated pricing. The aerial confirms a pool (+$62.00) and a waterfront parcel with dock/pier (+$87.00), both of which add measurable field complexity. No FEMA flood zone data was provided so no Elevation Certificate is included; lot size at 0.20-0.24 acres stays below the 0.31-acre threshold so no lot-size upcharge applies. No legal description is available at quote stage but this does not block pricing \u2014 if metes-and-bounds is confirmed on the legal description at order completion, a +$100.00 upcharge should be revisited.", "confidence": "MEDIUM", "escalate_flag": false, "escalate_reason": null, "flags": ["No legal description on file \u2014 if property is metes-and-bounds rather than platted lot-and-block, an additional +$100.00 complexity upcharge should be applied at order confirmation.", "No FEMA flood zone provided \u2014 given the coastal/waterfront location in Charlotte County, this property is likely in a flood zone (AE or VE). If an Elevation Certificate is required or requested, add $275.00 (plus $50.00 if Zone VE) as a separate line item.", "No parcel ID or legal description available at quote stage; surveyor should verify parcel boundaries via Charlotte County Property Appraiser prior to fieldwork.", "Aerial analysis confidence is LOW \u2014 field conditions (vegetation, storm damage noted in area) may reveal additional complexity not visible from satellite imagery."]}</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202606241704484826, "created_at": "2026-06-24T17:04:48", "customer_email": "nfroio@networkcraze.com", "customer_id": 202606241704484925, "customer_name": "Nick Froio", "customer_type": "individual", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": null, "invoiced": false, "order_id": 1000285867, "paid": false, "property_address": "261 BOCILLA DR", "property_city": "PLACIDA", "property_county": "CHARLOTTE COUNTY", "property_lat": "26.8631613", "property_lng": "-82.3132696", "property_state": "FLORIDA", "property_zip": "33946", "service_type": "Land Survey Only", "special_pricing": false, "status": "Quote", "status_code": 12, "updated_at": "2026-06-24T17:42:22"}, "ftf_customer": {"data": {"company_id": 202606241704484826, "company_name": "Nick Froio", "created_at": null, "custom_rate": null, "customer_id": 202606241704484925, "customer_type": "individual", "email": "nfroio@networkcraze.com", "first_name": "Nick Froio", "last_name": " ", "phone": "315-447-8788", "pricing_type": 0, "special_pricing": false}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": null, "source_url": "https://www.ccappraiser.com/Show_parcel.asp?acct=", "confidence": "LOW", "error": "Appraiser site unreachable (possible broken URL): https://www.ccappraiser.com/Show_parcel.asp?acct="}, "aerial_analysis": {"lot_shape": "rectangular", "estimated_lot_size": "~0.20 acres", "main_structure_footprint_sqft": 1400, "visible_structures": ["main house", "pool", "dock/pier"], "driveway_count": 1, "pool_visible": true, "apparent_encroachments": "null", "access_type": "street", "site_notes": "Property appears to be waterfront on the western side with a dock/pier extending into what appears to be a canal or bay. Coastal/waterfront location suggests flood zone and elevation certificate requirements likely applicable. Vegetation density on surrounding parcels may complicate boundary visibility. Road (Bocilla Dr) runs along eastern edge of parcel. Neighboring structures are closely spaced. Storm damage or vegetation disturbance visible in the area.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Nick Froio", "confidence": "HIGH"}, "client_email": {"value": "nfroio@networkcraze.com", "confidence": "HIGH"}, "property_address": {"value": "261 Bocilla Dr, Placida, FL 33946", "confidence": "HIGH"}, "property_county": {"value": "Charlotte County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated as 'Land Survey Only' in order data; no additional services indicated"}, "special_requirements": {"value": null, "confidence": "LOW"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features available; county appraiser site unreachable and no emails or aerial data provided"}, "client_tier": {"value": "residential", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Parcel ID / account number \u2014 county appraiser site unreachable", "Legal description \u2014 not available from any source", "Lot size \u2014 not available from any source", "Structure square footage \u2014 not available", "Property features (pool, shed, fence, driveway, etc.) \u2014 no aerial or appraiser data", "Special requirements or client notes \u2014 none provided", "Fieldwork date not yet scheduled", "Invoice not yet created and order not yet paid", "Flood zone determination pending"], "summary": "Individual residential client Nick Froio has submitted a quote-stage Land Survey Only order for a property at 261 Bocilla Dr, Placida, FL (Charlotte County), with no parcel data, legal description, or property details currently available."}}</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1000285867</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:28:42.842698+00:00</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-25 05:35 EDT</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>624</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:35:28.729869+00:00</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:03.935327+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1000285863</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>kimberly.nickens@onerealtitle.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Kimberly Nickens</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>5565 Silver Sun Dr, Apollo Beach, FL 33572</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>{"total_amount": 300.0, "services": [{"name": "Land Survey (Boundary)", "description": "Boundary/land survey for LOT 13, BLOCK 88, WATERSET PHASE 5A-1, 5565 Silver Sun Dr, Apollo Beach, FL 33572 (Hillsborough County). Plat-based survey of a small rectangular lot (~0.14 ac per DB, ~0.06 ac per aerial) within a dense townhouse development. FEMA Zone X \u2014 no elevation certificate required. Negotiated flat rate applied per management agreement with One Real Title.", "amount": 300.0}], "pricing_reasoning": "This is a straightforward Land Survey Only order for a small residential lot in Hillsborough County. The property is in FEMA Zone X, so no Elevation Certificate is needed. The client (One Real Title / WHBK Closing Services) has a management-approved negotiated rate of $300.00, which is applied as the flat total. No complexity upcharges are warranted: lot is sub-0.31 acres (no size upcharge), no pool, no waterfront, no metes-and-bounds description (plat-based), no Monroe County, and no heavy vegetation \u2014 the aerial shows a standard dense townhouse development reliant on recorded plat documents, which is routine for this property type.", "confidence": "HIGH", "escalate_flag": false, "escalate_reason": null, "flags": ["AERIAL_LOT_SIZE_DISCREPANCY: Database reports 0.14 acres; aerial analysis estimates ~0.06 acres. Likely reflects platted lot boundary vs. visible footprint in dense attached/townhouse layout. Neither value triggers a lot-size upcharge. No pricing impact.", "AERIAL_CONFIDENCE_LOW: Aerial analysis confidence is LOW due to dense attached townhouse construction making individual lot boundaries difficult to distinguish. Surveyor should rely on recorded plat (PB 132, PG 120) for boundary control.", "MULTIPLE_CERTIFICATIONS: Invoice certifies to KAREN BISHOP, JEFFREY P. BISHOP, ORTFL - ONE REAL TITLE OF FLORIDA LLC, and SEMINOLE MONEYTREE INC. Confirm all certification parties are acceptable under NexGen's standard practice before fieldwork.", "ZERO_ORDER_HISTORY: This client (One Real Title / WHBK Closing Services) has 0 prior orders with NexGen. Rate is validated via management-approved negotiated agreement \u2014 not inferred from order history."]}</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202503061903151302, "created_at": "2026-06-24T16:46:40", "customer_email": "kimberly.nickens@onerealtitle.com", "customer_id": 202507031713582437, "customer_name": "Kimberly  Nickens", "customer_type": "b2b", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12057C0515H\nZONE: X\nEFF: 08/28/2008", "invoiced": false, "order_id": 1000285863, "paid": false, "property_address": "5565 SILVER SUN DR", "property_city": "APOLLO BEACH", "property_county": "HILLSBOROUGH COUNTY", "property_lat": "27.7589142", "property_lng": "-82.373576", "property_state": "FL", "property_zip": "33572", "service_type": "Land Survey Only", "special_pricing": true, "status": "Pending", "status_code": 1, "updated_at": "2026-06-24T16:59:36"}, "ftf_customer": {"data": {"company_id": 202503061903151302, "company_name": "WHBK Closing Services, LLC DBA One Real Title", "created_at": null, "custom_rate": 300.0, "customer_id": 202507031713582437, "customer_type": "b2b", "email": "kimberly.nickens@onerealtitle.com", "first_name": "Kimberly ", "last_name": "Nickens", "phone": "8135689197", "pricing_type": 0, "special_pricing": true}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "Property search page for 5565 Silver Sun Dr, Hillsborough County, FL returned no data. The page text contains only the website UI framework and no actual parcel record data was loaded or returned for this address.", "source_url": "https://gis.hcpafl.org/propertysearch?address=5565%20SILVER%20SUN%20DR", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "rectangular", "estimated_lot_size": "~0.06 acres", "main_structure_footprint_sqft": 1400, "visible_structures": ["main house/townhouse unit", "shared driveway/parking area"], "driveway_count": 1, "pool_visible": false, "apparent_encroachments": null, "access_type": "shared", "site_notes": "Property appears to be part of a dense townhouse/condominium development with uniform row units oriented diagonally along a central pedestrian corridor. Lot boundaries are difficult to distinguish individually due to attached/semi-attached construction style. Shared driveways and parking areas are evident. A diagonal road/pathway bisects the development. Boundary survey would need to rely heavily on recorded plat documents. Units appear to share walls and common areas, suggesting HOA or condominium regime.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Kimberly Nickens", "confidence": "HIGH"}, "client_email": {"value": "kimberly.nickens@onerealtitle.com", "confidence": "HIGH"}, "property_address": {"value": "5565 Silver Sun Dr, Apollo Beach, FL 33572", "confidence": "HIGH"}, "property_county": {"value": "Hillsborough County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated as 'Land Survey Only'; no elevation certificate requested."}, "special_requirements": {"value": "Special pricing applies; custom rate of $300.00 on file for this B2B client.", "confidence": "HIGH"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features available; no emails, attachments, or additional data sources provided."}, "client_tier": {"value": "b2b", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Lot size unknown \u2014 not provided in any data source", "Legal description not provided", "Structure square footage unknown", "Property features unknown (pool, shed, fencing, driveways, etc.)", "No fieldwork date scheduled yet", "No emails or attachments found to supplement order details", "Urgency not explicitly stated \u2014 assumed normal"], "summary": "B2B land survey order for Kimberly Nickens of One Real Title at 5565 Silver Sun Dr, Apollo Beach, FL 33572 (Hillsborough County) with a special custom rate of $300.00, currently pending with no fieldwork scheduled."}}</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>1000285863</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:29:15.679056+00:00</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-25 05:35 EDT</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>300</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:35:55.322843+00:00</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:04.055328+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1000285860</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>condo_rejected</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>kali@mondocklaw.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Kali Peley</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>801 River Point Dr, Naples, FL 34102</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>{"total_amount": 0.0, "services": [], "pricing_reasoning": "Condo/unit order \u2014 unit number 'Boat slip 62' detected in ng_unit_number", "confidence": "N/A", "escalate_flag": true, "escalate_reason": "Condo/unit order \u2014 unit number 'Boat slip 62' detected in ng_unit_number", "flags": ["condo_rejected"]}</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202111241424361546, "created_at": "2026-06-24T16:36:40", "customer_email": "kali@mondocklaw.com", "customer_id": 202411051555164447, "customer_name": "Kali  Peley", "customer_type": "b2b", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": null, "invoiced": false, "order_id": 1000285860, "paid": false, "property_address": "801 RIVER POINT DR", "property_city": "NAPLES", "property_county": "Collier County", "property_lat": "26.1399871", "property_lng": "-81.7883738", "property_state": "FLORIDA", "property_zip": "34102", "service_type": "Land Survey Only", "special_pricing": true, "status": "Quote", "status_code": 12, "updated_at": "2026-06-24T16:40:46"}, "ftf_customer": {"data": {"company_id": 202111241424361546, "company_name": "Mondock Law PLLC", "created_at": null, "custom_rate": 450.0, "customer_id": 202411051555164447, "customer_type": "b2b", "email": "kali@mondocklaw.com", "first_name": " Kali ", "last_name": "Peley", "phone": "2396732211", "pricing_type": 0, "special_pricing": true}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "Page unavailable at time of request. No property data could be retrieved from the Collier County Property Appraiser website for 801 River Point Dr.", "source_url": "https://www.collierappraiser.com/search?address=801%20RIVER%20POINT%20DR", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "irregular", "estimated_lot_size": "~1.5 acres", "main_structure_footprint_sqft": 8500, "visible_structures": ["multi-unit residential or condominium building", "marina dock structures", "boat slips", "parking areas", "secondary commercial/storage buildings nearby"], "driveway_count": 2, "pool_visible": false, "apparent_encroachments": "Boat slips and dock structures extend into the waterway; boundary between upland property and riparian/water rights area may require clarification. Adjacent red-roofed commercial structures appear in close proximity and may share access.", "access_type": "street", "site_notes": "Property appears to be a waterfront marina condominium complex with multiple boat slips along interior canal. Riparian rights and water boundary delineation will be critical for this survey. Dock fingers extend significantly into the canal. Shared access with adjacent commercial parcels is possible. Elevation certificate likely required given waterfront/coastal proximity. Multiple structures visible on or near apparent parcel boundaries. Confirm limits of upland vs. submerged land ownership.", "confidence": "MEDIUM"}, "packet": {"client_name": {"value": "Kali Peley", "confidence": "HIGH"}, "client_email": {"value": "kali@mondocklaw.com", "confidence": "HIGH"}, "property_address": {"value": "801 River Point Dr, Naples, FL 34102", "confidence": "HIGH"}, "property_county": {"value": "Collier County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated as Land Survey Only; however, aerial analysis suggests riparian/water boundary delineation and possible elevation certificate may also be needed \u2014 not yet ordered."}, "special_requirements": {"value": "Waterfront marina condominium complex; riparian rights and water boundary delineation critical; dock fingers extend into canal; upland vs. submerged land ownership limits must be confirmed; possible shared access with adjacent commercial parcels.", "confidence": "MEDIUM"}, "lot_size": {"value": "~1.5 acres", "confidence": "MEDIUM"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": 8500, "confidence": "MEDIUM"}, "property_features": {"value": {"multi_unit_residential_or_condo_building": true, "marina_dock_structures": true, "boat_slips": true, "parking_areas": true, "secondary_commercial_storage_buildings_nearby": true, "pool": false, "driveway_count": 2, "waterfront": true, "irregular_lot": true}, "confidence": "MEDIUM", "notes": "All features derived from aerial image analysis at medium confidence; no pool visible; boat slips and dock structures extend into adjacent waterway."}, "client_tier": {"value": "b2b", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "mixed", "gaps": ["Legal description not provided \u2014 required for survey", "Parcel ID / folio number not provided", "Limits of upland vs. submerged land ownership not confirmed", "Riparian rights scope not defined \u2014 client has not explicitly ordered water boundary delineation", "Elevation certificate not ordered but may be warranted given coastal/waterfront location \u2014 needs client clarification", "Fieldwork date not scheduled", "Invoice not yet generated and order is still in Quote status", "Custom rate of $450 noted \u2014 confirm if this applies to all services or base survey only", "Shared access with adjacent commercial parcels needs confirmation", "No matching emails found \u2014 no additional context from client communications"], "summary": "B2B land survey order for Mondock Law PLLC at a waterfront marina condominium complex in Naples, FL, currently in Quote status, with critical unresolved questions around riparian boundaries, submerged land ownership, and potential elevation certificate requirements."}}</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:29:49.709782+00:00</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:36:03.133762+00:00</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:36:03.142528+00:00</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:04.176127+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1000285856</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>corrine@insured-title.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Corrine Kent</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>3131 N BLVD &amp; 3112 WOODROW AVE (VACANT LOT), TAMPA, FL 33603</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>{"total_amount": 512.0, "services": [{"name": "Land Survey (Boundary)", "description": "Boundary survey for combined vacant lot parcels at 3131 N Blvd &amp; 3112 Woodrow Ave, Hillsborough County. Negotiated B2B rate for Insured Title Agency LLC (OLD_TITLE client). Certifications to: KINDE LLC, Insured Title Agency, Fifth Third Bank N.A., and Commonwealth Land Title Insurance Company.", "amount": 450.0}, {"name": "Lot Size Complexity Upcharge (0.31\u20130.50 ac)", "description": "Combined parcel is approximately 0.34\u20130.35 acres per DB and aerial analysis, placing it in the 0.31\u20130.50 ac upcharge tier. Additionally, the legal description covers four separate lots across two blocks (Lots 4, 5, 6 Block 1 and Lot 5 Block 2), increasing field and office complexity. The partial demolition/construction activity and unclear boundary delineation between the two addresses further support this upcharge.", "amount": 62.0}], "pricing_reasoning": "The negotiated rate of $450.00 is honored per management agreement with Insured Title Agency LLC (OLD_TITLE client tier). A lot size upcharge of $62.00 is applied because the combined parcel falls in the 0.31\u20130.50 ac tier and the legal description spans four lots across two blocks with an ambiguous boundary between the two addresses \u2014 aerial imagery confirms unclear delineation, partial demolition debris, and dual street frontage, all of which add legitimate field complexity. No EC is ordered (Zone X, no flood certificate requested), no pool, no waterfront, no Monroe County, and no metes-and-bounds description (plat-referenced legal), so no additional upcharges are warranted.", "confidence": "MEDIUM", "escalate_flag": false, "escalate_reason": null, "flags": ["MULTI-PARCEL: Legal description covers four lots across two blocks and two street addresses \u2014 field crew should confirm parcel boundaries carefully before staking.", "AERIAL CONFIDENCE LOW: Satellite imagery shows partially demolished or gutted structure on 3131 N Blvd with debris; boundary between the two parcels is unclear from aerial. Field crew should exercise caution and verify legal corners.", "DUAL CERTIFICATION: Four parties named as certificate holders (KINDE LLC, Insured Title Agency, Fifth Third Bank N.A., Commonwealth Land Title Insurance). Confirm all certificate language is approved before delivery.", "COMMERCIAL FLAG FALSE BUT STRUCTURE PRESENT: Aerial shows a large commercial/industrial building footprint (~4,800 sqft) despite commercial_flag=False and a vacant lot designation. This may affect scope if as-built or improvement location is later requested.", "QUOTE STATUS: Order notes indicate job is pending fieldwork scheduling and was quoted at $450 special pricing \u2014 total here reflects $450 base + justified complexity upcharge of $62."]}</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 201801311051487027, "created_at": "2026-06-24T16:04:32", "customer_email": "corrine@insured-title.com", "customer_id": 202212271434085171, "customer_name": "Corrine  Kent", "customer_type": "b2b", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12057C0352J\nZONE:X\nEFF: 10/07/2021", "invoiced": false, "order_id": 1000285856, "paid": false, "property_address": "3131 N BLVD &amp; 3112 WOODROW AVE(VACANT LOT)", "property_city": "TAMPA", "property_county": "HILLSBOROUGH COUNTY", "property_lat": "27.9725722", "property_lng": "-82.46742979999999", "property_state": "FL", "property_zip": "33603", "service_type": "Land Survey Only", "special_pricing": true, "status": "Quote", "status_code": 12, "updated_at": "2026-06-24T19:33:15"}, "ftf_customer": {"data": {"company_id": 201801311051487027, "company_name": "Insured Title Agency LLC", "created_at": null, "custom_rate": 450.0, "customer_id": 202212271434085171, "customer_type": "b2b", "email": "corrine@insured-title.com", "first_name": "Corrine ", "last_name": "Kent", "phone": "8138553585", "pricing_type": 0, "special_pricing": true}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "Property address: 3131 N BLVD &amp; 3112 WOODROW AVE (VACANT LOT), Hillsborough County, FL. The page did not return any search results or parcel data. The property is noted as a vacant lot. No folio number, legal description, lot size, or other data was available from the page content provided.", "source_url": "https://gis.hcpafl.org/propertysearch?address=3131%20N%20BLVD%20%26%203112%20WOODROW%20AVE%28VACANT%20LOT%29", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "rectangular", "estimated_lot_size": "~0.35 acres (combined parcels)", "main_structure_footprint_sqft": 4800, "visible_structures": ["commercial/industrial building (partially demolished or under construction)", "paved parking area", "vacant lot area"], "driveway_count": 2, "pool_visible": false, "apparent_encroachments": "Possible debris or demolition materials visible on structure footprint; unclear boundary between 3131 N Blvd and 3112 Woodrow Ave vacant lot", "access_type": "street", "site_notes": "Property appears to consist of a partially demolished or gutted commercial structure on 3131 N Blvd with an adjacent vacant lot at 3112 Woodrow Ave. The main building shows significant roof damage or removal visible from aerial. Corner/dual-street access from N Blvd and Woodrow Ave. Paved parking lot visible to the east of structure. Boundary delineation between the two parcels is critical for survey. Potential utility lines visible along N Blvd corridor. Surrounding area is residential with scattered commercial uses.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Corrine Kent", "confidence": "HIGH"}, "client_email": {"value": "corrine@insured-title.com", "confidence": "HIGH"}, "property_address": {"value": "3131 N BLVD &amp; 3112 WOODROW AVE (VACANT LOT), TAMPA, FL 33603", "confidence": "HIGH"}, "property_county": {"value": "Hillsborough County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated as 'Land Survey Only'; no additional services indicated. Vacant lot noted \u2014 no elevation certificate requested."}, "special_requirements": {"value": "Special pricing applies per customer account (custom rate: $450.00)", "confidence": "HIGH"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "HIGH"}, "property_features": {"value": {"vacant_lot": true, "structures": false, "pool": null, "shed": null, "driveway": null}, "confidence": "MEDIUM", "notes": "Property is explicitly noted as a vacant lot; no structures expected but no site visit or aerial data confirmed. Pool, shed, and driveway unknown."}, "client_tier": {"value": "b2b", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Lot size not provided \u2014 needed for accurate scoping and pricing", "Legal description not provided \u2014 required for survey work on a vacant lot", "Two addresses listed (3131 N BLVD &amp; 3112 WOODROW AVE) \u2014 confirm if this is one combined parcel or two separate lots", "No fieldwork date scheduled (fieldwork_at is null)", "Order has not been invoiced or paid \u2014 still in Quote status", "No matching emails found \u2014 no additional context or client instructions available", "Property features entirely unknown \u2014 confirm vacancy and absence of encroachments or easements", "Urgency not communicated \u2014 no rush flag or deadline specified"], "summary": "B2B land survey order for Corrine Kent of Insured Title Agency LLC covering a vacant lot at two adjacent addresses in Tampa, FL (Hillsborough County), currently in Quote status with special pricing at $450 and pending fieldwork scheduling."}}</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1000285856</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:30:24.857534+00:00</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-25 05:36 EDT</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>512</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:36:39.174775+00:00</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:04.296191+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1000285853</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>details_missing</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>kimberly@collinbuilders.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kimberly Boyle </t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>321 RILYN DR</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:31:04.968919+00:00</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:31:04.982048+00:00</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:04.377383+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1000285842</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>elisha@rackelectric.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Elisha Smallwood</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>5812 Lady Luck Rd, Palm Beach Gardens, FL 33418</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>{"total_amount": 725.0, "services": [{"name": "Land Survey (Base Rate)", "description": "Negotiated base survey rate for Rack Electric LLC (OLD_TITLE client tier), as agreed upon by management.", "amount": 450.0}, {"name": "Lot Size Complexity Upcharge (1.01\u20132.00 ac)", "description": "Aerial analysis estimates ~1.5 acres (DB shows 1.14 ac), both figures fall within the 1.01\u20132.00 ac complexity tier, warranting the standard upcharge for larger residential estate parcels.", "amount": 275.0}], "pricing_reasoning": "The base survey rate of $450.00 is the management-agreed negotiated rate for Rack Electric LLC and is used as-is. The lot size of ~1.14\u20131.5 acres (DB and aerial estimates both confirm the 1.01\u20132.00 ac tier) triggers a $275.00 complexity upcharge. No Elevation Certificate was ordered (FEMA Zone X, no flood insurance driver), so no EC line item applies. Pool visibility and possible drainage/water channel along the western edge were considered: the pool upcharge (+$62) and waterfront/canal upcharge (+$87) were evaluated but not applied \u2014 the pool is a standard estate amenity and the western water feature appears to be a drainage swale or easement rather than a true navigable canal, and the client tier rate already reflects a discounted structure that absorbs minor site features. Heavy vegetation along the western boundary and mature tree canopy may slow fieldwork but do not rise to a standalone upcharge given the negotiated pricing framework in place.", "confidence": "MEDIUM", "escalate_flag": false, "escalate_reason": null, "flags": ["Lot size discrepancy: DB records show 1.14 ac while aerial analysis estimates ~1.5 ac \u2014 both fall within the same complexity tier (1.01\u20132.00 ac) so pricing is unaffected, but field crew should verify true parcel boundaries.", "Western boundary: mature tree canopy and possible drainage easement or water channel may obscure monuments \u2014 crew should be advised to allocate additional time for boundary recovery in that area.", "No legal description text was provided in the order; if the parcel is metes-and-bounds rather than a platted lot-and-block, a +$100.00 metes-and-bounds upcharge may need to be revisited after legal description is confirmed.", "Order count for Rack Electric LLC is 0 \u2014 this is their first order with NexGen despite being classified OLD_TITLE; confirm negotiated rate authorization with management before finalizing invoice."]}</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202412091849570674, "created_at": "2026-06-24T14:10:51", "customer_email": "elisha@rackelectric.com", "customer_id": 202510162051204016, "customer_name": "Elisha  Smallwood", "customer_type": "b2b", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12099C0367F\nZONE:X\nEFF: 10/05/2017", "invoiced": false, "order_id": 1000285842, "paid": false, "property_address": "5812 LADY LUCK RD", "property_city": "PALM BEACH GARDENS", "property_county": "Palm Beach County", "property_lat": "26.8011155", "property_lng": "-80.1281192", "property_state": "FLORIDA", "property_zip": "33418", "service_type": "Land Survey Only", "special_pricing": true, "status": "Quote", "status_code": 12, "updated_at": "2026-06-24T14:26:50"}, "ftf_customer": {"data": {"company_id": 202412091849570674, "company_name": "Rack Electric LLC", "created_at": null, "custom_rate": 450.0, "customer_id": 202510162051204016, "customer_type": "b2b", "email": "elisha@rackelectric.com", "first_name": "Elisha ", "last_name": "Smallwood", "phone": "5618730906", "pricing_type": 0, "special_pricing": true}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "No property-specific data was returned in the page text. The page appears to show only the Palm Beach County PAO homepage/search interface without results for 5812 LADY LUCK RD. A direct lookup on pbcpao.gov is required to retrieve parcel details.", "source_url": "https://pbcpao.gov/?address=5812%20LADY%20LUCK%20RD", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "irregular", "estimated_lot_size": "~1.5 acres", "main_structure_footprint_sqft": 4800, "visible_structures": ["main house", "pool", "detached outbuilding or guest structure", "paved circular driveway area", "putting green or recreational lawn feature"], "driveway_count": 1, "pool_visible": true, "apparent_encroachments": "null", "access_type": "street", "site_notes": "Property appears to be a large residential estate lot with mature tree canopy along western boundary, which may obscure boundary markers. A water channel or drainage easement runs along the western edge. Multiple neighboring structures are in close proximity to the north and east, warranting careful boundary verification. Circular driveway layout suggests a curved easement or access apron at street frontage. The putting green-style feature in the rear yard should be noted for elevation survey purposes.", "confidence": "MEDIUM"}, "packet": {"client_name": {"value": "Elisha Smallwood", "confidence": "HIGH"}, "client_email": {"value": "elisha@rackelectric.com", "confidence": "HIGH"}, "property_address": {"value": "5812 Lady Luck Rd, Palm Beach Gardens, FL 33418", "confidence": "HIGH"}, "property_county": {"value": "Palm Beach County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated as 'Land Survey Only' in order data. No elevation certificate requested."}, "special_requirements": {"value": "Special pricing applies per customer profile (custom rate $450.00). Mature tree canopy along western boundary may obscure boundary markers. Water channel or drainage easement along western edge warrants field attention. Multiple neighboring structures in close proximity to north and east require careful boundary verification.", "confidence": "MEDIUM"}, "lot_size": {"value": "~1.5 acres", "confidence": "MEDIUM"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": 4800, "confidence": "MEDIUM"}, "property_features": {"value": {"pool": true, "detached_outbuilding_or_guest_structure": true, "circular_driveway": true, "putting_green_or_recreational_lawn": true, "water_channel_or_drainage_easement": true, "mature_tree_canopy_western_boundary": true}, "confidence": "MEDIUM", "notes": "All features derived from aerial image analysis at medium confidence. Pool, detached outbuilding, circular driveway, putting green, drainage easement, and tree canopy all noted. No physical site visit confirmed."}, "client_tier": {"value": "b2b", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "mixed", "gaps": ["Legal description not provided \u2014 needed for survey document preparation", "Fieldwork date not yet scheduled (fieldwork_at is null)", "Invoice not yet generated (invoiced = false)", "Order is still in Quote status \u2014 awaiting client confirmation", "No matching emails found \u2014 no additional context from client correspondence", "Nature of detached outbuilding or guest structure unconfirmed \u2014 may affect scope", "Drainage easement along western boundary not documented \u2014 recorded easement details needed", "Lot size is aerial estimate only (~1.5 acres) \u2014 legal lot dimensions not confirmed", "Purpose or end-use of survey not stated (e.g., permitting, title, construction)"], "summary": "B2B land survey order for Elisha Smallwood of Rack Electric LLC at a large residential estate parcel (~1.5 acres) in Palm Beach Gardens, FL, currently in Quote status with special pricing applied and pending fieldwork scheduling."}}</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1000285842</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:31:40.750757+00:00</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-25 05:37 EDT</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>725</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:37:07.210383+00:00</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:04.448941+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1000285807</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>mike@mikesilvermanart.com</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mike Silverman</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>3075 Riviera Drive, Delray Beach, FL 33445</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>{"total_amount": 537.0, "services": [{"name": "Land Survey (Boundary)", "description": "Base boundary/land survey rate for individual residential client in Palm Beach County.", "amount": 475.0}, {"name": "Lot Size Upcharge (0.31\u20130.50 ac)", "description": "Property is 0.33 acres, falling in the 0.31\u20130.50 ac complexity band. Upcharge applied per pricing guidelines.", "amount": 62.0}], "pricing_reasoning": "This is a standard residential boundary/land survey for an individual client (Mike Silverman) in Palm Beach County. The base rate for individual clients is $475.00. The lot size of 0.33 acres triggers the 0.31\u20130.50 ac upcharge of $62.00. FEMA Zone X requires no elevation certificate and carries no flood-zone upcharge. No pool, waterfront, metes-and-bounds, heavy vegetation, or Monroe County factors are supported by the available data. Aerial imagery was unavailable, so no additional complexity could be confirmed from that source, and no further upcharges are applied speculatively.", "confidence": "MEDIUM", "escalate_flag": false, "escalate_reason": null, "flags": ["Aerial imagery unavailable for this address \u2014 field crew should note any encroachments, access issues, or vegetation complexity on arrival; re-price if significant complexity is discovered in the field.", "Legal description was not provided in the order \u2014 crew should obtain and verify prior to fieldwork; metes-and-bounds description could trigger an additional $100.00 upcharge if applicable.", "First-time individual client with 0 prior orders; no negotiated rate applies."]}</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202606231901350939, "created_at": "2026-06-23T19:01:35", "customer_email": "mike@mikesilvermanart.com", "customer_id": 202606231901351042, "customer_name": "Mike Silverman", "customer_type": "individual", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12099C0976G\nZONE:X\nEFF: 12/20/2024", "invoiced": false, "order_id": 1000285807, "paid": false, "property_address": "3075 RIVIERA DRIVE", "property_city": "DELRAY BEACH", "property_county": "Palm Beach County", "property_lat": "26.4818743", "property_lng": "-80.10458589999999", "property_state": "FLORIDA", "property_zip": "33445", "service_type": "Land Survey Only", "special_pricing": false, "status": "Quote", "status_code": 12, "updated_at": "2026-06-23T19:32:27"}, "ftf_customer": {"data": {"company_id": 202606231901350939, "company_name": "Mike Silverman", "created_at": null, "custom_rate": null, "customer_id": 202606231901351042, "customer_type": "individual", "email": "mike@mikesilvermanart.com", "first_name": "Mike Silverman", "last_name": " ", "phone": "4254448020", "pricing_type": 0, "special_pricing": false}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "No property-specific data was returned in the page text. The page appears to have loaded the Palm Beach County PAO homepage rather than a specific property record for 3075 Riviera Drive. A manual search on https://pbcpao.gov may be required to retrieve parcel details.", "source_url": "https://pbcpao.gov/?address=3075%20RIVIERA%20DRIVE", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "other", "estimated_lot_size": null, "main_structure_footprint_sqft": null, "visible_structures": [], "driveway_count": null, "pool_visible": false, "apparent_encroachments": null, "access_type": "unclear", "site_notes": "No aerial imagery available for this location. The map tile returned an error stating 'Sorry, we have no imagery here.' No property analysis can be performed. Manual field survey or alternative imagery source required for 3075 Riviera Drive.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Mike Silverman", "confidence": "HIGH"}, "client_email": {"value": "mike@mikesilvermanart.com", "confidence": "HIGH"}, "property_address": {"value": "3075 Riviera Drive, Delray Beach, FL 33445", "confidence": "HIGH"}, "property_county": {"value": "Palm Beach County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated as 'Land Survey Only'; no elevation certificate required per elevation_cert flag"}, "special_requirements": {"value": null, "confidence": "LOW"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features available; no emails, attachments, or appraisal data found to infer features such as pool, shed, or structures"}, "client_tier": {"value": "residential", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Lot size unknown \u2014 needed for accurate quoting", "Legal description not provided", "Structure square footage unknown", "Property features (pool, shed, fence, driveway, etc.) unknown \u2014 no site visit or supporting documents yet", "Special requirements or access instructions not provided", "No emails found to supplement order details", "Invoice not yet created and estimate not yet sent \u2014 pricing pending"], "summary": "Individual residential client Mike Silverman is requesting a Land Survey Only for a property at 3075 Riviera Drive, Delray Beach, FL 33445 (Palm Beach County), currently in Quote status with no fieldwork scheduled and key property details still needed."}}</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1000285807</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:32:10.312490+00:00</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-06-25 05:37 EDT</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>537</v>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:37:30.775361+00:00</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:25:04.513409+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: drain batch 2 of recent invoice-needed orders to sheet (18 total)
Ran A1->A2->A3 locally again (DB reachable from here). Sheet now holds 18 real,
correctly-priced orders. State committed so CI dedups. NOTE: REST intake validated
unsafe (89% false positives vs ng_invoice_needed) so intake stays MySQL-only.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/invoice_pipeline_state.xlsx
+++ b/data/invoice_pipeline_state.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1222,6 +1222,682 @@
       <c r="V11" t="inlineStr">
         <is>
           <t>2026-06-25T09:25:04.513409+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1000285785</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>delivered_flagged</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>karylindgren@gmail.com</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Kary Lindgren</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2729 NE 22nd Ave, Lighthouse Point, FL 33064</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202606231706008328, "created_at": "2026-06-23T17:09:59", "customer_email": "karylindgren@gmail.com", "customer_id": 202606231706011220, "customer_name": "Kary lindgren", "customer_type": "individual", "delivered_at": "2026-06-24T18:21:07", "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12011C0189J\nZONE: AE\nELEV: 07 FT\nEFF: 07/31/2024", "invoiced": false, "order_id": 1000285785, "paid": true, "property_address": "2729 NE 22ND AVE", "property_city": "LIGHTHOUSE POINT", "property_county": "Broward County", "property_lat": "26.2646984", "property_lng": "-80.0934956", "property_state": "FL", "property_zip": "33064", "service_type": "Land Survey Only", "special_pricing": true, "status": "Delivered", "status_code": 8, "updated_at": "2026-06-24T18:22:04"}, "ftf_customer": {"data": {"company_id": 202606231706008328, "company_name": "Kary lindgren", "created_at": null, "custom_rate": 300.0, "customer_id": 202606231706011220, "customer_type": "individual", "email": "karylindgren@gmail.com", "first_name": "Kary", "last_name": "lindgren", "phone": "3107027900", "pricing_type": 0, "special_pricing": true}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": null, "source_url": "https://web.bcpa.net/bcpaclient/#/Record-Search?fnumber=", "confidence": "LOW", "error": "Appraiser site unreachable (possible broken URL): https://web.bcpa.net/bcpaclient/#/Record-Search?fnumber="}, "aerial_analysis": {"lot_shape": "rectangular", "estimated_lot_size": "~0.25 acres", "main_structure_footprint_sqft": 2200, "visible_structures": ["main house", "pool", "patio/deck area"], "driveway_count": 1, "pool_visible": true, "apparent_encroachments": "Mature tree canopy from adjacent properties may overhang lot boundaries; precise boundary determination obscured by dense vegetation", "access_type": "street", "site_notes": "Property appears to be located on a residential block between a north-south running road (west side) and a parallel arterial road to the east. Dense tropical vegetation surrounds the structure making boundary corner identification difficult from aerial view. Pool is located on the south or west side of main structure. Neighboring structures are in close proximity, warranting careful boundary verification. Low-lying Florida coastal area suggests elevation certificate may be relevant.", "confidence": "MEDIUM"}, "packet": {"client_name": {"value": "Kary Lindgren", "confidence": "HIGH"}, "client_email": {"value": "karylindgren@gmail.com", "confidence": "HIGH"}, "property_address": {"value": "2729 NE 22nd Ave, Lighthouse Point, FL 33064", "confidence": "HIGH"}, "property_county": {"value": "Broward County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated as 'Land Survey Only'; no elevation certificate requested despite property being in FEMA Flood Zone AE"}, "special_requirements": {"value": "Special pricing applied (custom rate $300.00); Flood Zone AE \u2014 Panel 12011C0189J, base flood elevation 7 ft, effective 07/31/2024; dense tropical vegetation may complicate boundary corner identification", "confidence": "MEDIUM"}, "lot_size": {"value": "~0.25 acres", "confidence": "MEDIUM"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": 2200, "confidence": "MEDIUM"}, "property_features": {"value": {"pool": true, "patio_deck": true, "driveway_count": 1, "main_house": true, "lot_shape": "rectangular", "vegetation": "dense tropical canopy"}, "confidence": "MEDIUM", "notes": "Pool, patio/deck, and single driveway identified via aerial analysis; no shed or outbuildings noted; mature tree canopy from adjacent properties may overhang boundaries"}, "client_tier": {"value": "residential", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "mixed", "gaps": ["Legal description not available \u2014 county property appraiser site unreachable", "Parcel/folio number unknown \u2014 appraiser lookup failed", "Exact lot size unconfirmed \u2014 aerial estimate only (~0.25 acres)", "No matching emails found \u2014 no additional client instructions or context available", "Fieldwork date not yet scheduled (fieldwork_at is null)", "Elevation certificate not ordered despite Flood Zone AE designation \u2014 confirm client is aware", "Structure square footage is an aerial estimate only \u2014 not verified by appraiser or MLS data", "Presence of any easements, encroachments, or encumbrances unknown without legal description or appraiser data"], "summary": "Residential land survey only for Kary Lindgren at 2729 NE 22nd Ave, Lighthouse Point, FL (Broward County), delivered under special pricing ($300), located in FEMA Flood Zone AE with dense vegetation that may complicate boundary identification; legal description and parcel data unavailable due to appraiser site failure."}}</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:35:17.683586+00:00</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:42:09.744423+00:00</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:42:09.754974+00:00</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:15.952024+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1000285776</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>digiconconstruction@gmail.com</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Digicon LLC</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2105 NE 62ND ST, FORT LAUDERDALE, FL 33308</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>{"total_amount": 462.0, "services": [{"name": "Land Survey (Boundary)", "description": "Base boundary survey for residential lot at 2105 NE 62ND ST, Fort Lauderdale, Broward County. Old Title client base rate applied.", "amount": 400.0}, {"name": "Pool Complexity Upcharge", "description": "Pool is confirmed visible in aerial imagery in the rear/side yard. Pool structures require additional corner and setback verification during field work.", "amount": 62.0}], "pricing_reasoning": "This is a standard boundary survey (Land Survey Only) for a residential property in Broward County. The client Digicon LLC is classified as OLD_TITLE with a default base rate of $400.00. No Elevation Certificate was requested, so the $275.00 EC line item is not applicable. The lot is approximately 0.18\u20130.20 acres, which falls under the 0.31-acre threshold, so no lot-size upcharge applies. A pool is clearly confirmed in the aerial imagery and noted in the order notes, justifying the $62.00 pool upcharge. No waterfront, metes-and-bounds description, Monroe County location, or heavy vegetation conditions were identified that would warrant additional upcharges \u2014 while mature tree canopy is noted, it does not rise to the level of 'heavy vegetation' warranting the $112 flag. No legal description was provided, but the parcel appears to be a platted lot rather than a metes-and-bounds description, so no M&amp;B upcharge is applied.", "confidence": "MEDIUM", "escalate_flag": false, "escalate_reason": null, "flags": ["No legal description provided in order \u2014 assumed platted lot based on aerial and order context. Recommend confirming with county records before fieldwork.", "County appraiser data noted as currently unavailable per order notes \u2014 lot size and parcel details rely on aerial estimate (~0.20 ac) and DB value (0.18 ac). Both are below the 0.31-acre upcharge threshold so no material pricing impact.", "No prior order history for Digicon LLC with NexGen (0 orders). Default OLD_TITLE rate of $400.00 applied per guidelines."]}</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202606231600523269, "created_at": "2026-06-23T16:00:52", "customer_email": "digiconconstruction@gmail.com", "customer_id": 202606231600523371, "customer_name": "Digicon LLC", "customer_type": "b2b", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12011C0378J\nZONE:AE\nEFF: 07/31/2024", "invoiced": false, "order_id": 1000285776, "paid": false, "property_address": "2105 NE 62ND ST", "property_city": "FORT LAUDERDALE", "property_county": "Broward County", "property_lat": "26.2038641", "property_lng": "-80.11754309999999", "property_state": "FLORIDA", "property_zip": "33308", "service_type": "Land Survey Only", "special_pricing": false, "status": "Quote", "status_code": 12, "updated_at": "2026-06-23T16:38:20"}, "ftf_customer": {"data": {"company_id": 202606231600523269, "company_name": "Digicon LLC", "created_at": null, "custom_rate": null, "customer_id": 202606231600523371, "customer_type": "b2b", "email": "digiconconstruction@gmail.com", "first_name": "Digicon LLC", "last_name": " ", "phone": "5142160598", "pricing_type": 0, "special_pricing": false}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": null, "source_url": "https://web.bcpa.net/bcpaclient/#/Record-Search?fnumber=", "confidence": "LOW", "error": "Appraiser site unreachable (possible broken URL): https://web.bcpa.net/bcpaclient/#/Record-Search?fnumber="}, "aerial_analysis": {"lot_shape": "rectangular", "estimated_lot_size": "~0.20 acres", "main_structure_footprint_sqft": 1800, "visible_structures": ["main house", "pool", "patio/deck area"], "driveway_count": 1, "pool_visible": true, "apparent_encroachments": null, "access_type": "street", "site_notes": "Property appears to be a mid-block residential lot in a dense suburban neighborhood. Pool is visible in the rear/side yard. Surrounding lots have similar dimensions and configurations. Mature tree canopy present which may obscure boundary corners. Street-facing frontage appears consistent with neighboring parcels. No obvious encroachments or easement conflicts visible from aerial perspective.", "confidence": "MEDIUM"}, "packet": {"client_name": {"value": "Digicon LLC", "confidence": "HIGH"}, "client_email": {"value": "digiconconstruction@gmail.com", "confidence": "HIGH"}, "property_address": {"value": "2105 NE 62ND ST, FORT LAUDERDALE, FL 33308", "confidence": "HIGH"}, "property_county": {"value": "Broward County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly listed as 'Land Survey Only'; no additional services requested. Property is in Flood Zone AE \u2014 elevation certificate not ordered but may be relevant."}, "special_requirements": {"value": null, "confidence": "LOW"}, "lot_size": {"value": "~0.20 acres", "confidence": "MEDIUM"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": 1800, "confidence": "MEDIUM"}, "property_features": {"value": {"pool": true, "driveway_count": 1, "patio_deck": true, "main_house": true, "encroachments": false, "mature_trees": true}, "confidence": "MEDIUM", "notes": "All features derived from aerial image analysis at medium confidence. Pool visible in rear/side yard. Mature tree canopy may obscure boundary corners. No shed detected."}, "client_tier": {"value": "b2b", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "mixed", "gaps": ["Legal description not available \u2014 county appraiser site unreachable", "Exact lot size not confirmed \u2014 appraiser data unavailable, aerial estimate only (~0.20 acres)", "No special requirements or notes provided by client", "Urgency not stated \u2014 assumed normal based on Quote status", "Structure square footage is aerial estimate only \u2014 no appraiser or permit data to confirm", "Elevation certificate not ordered but property is in Flood Zone AE \u2014 may warrant follow-up with client", "Fieldwork date not yet scheduled", "No matching emails found \u2014 no additional context from client communications"], "summary": "B2B client Digicon LLC has placed a Land Survey Only quote for a residential property at 2105 NE 62ND ST, Fort Lauderdale in Flood Zone AE, featuring a pool and estimated at ~0.20 acres, with county appraiser data currently unavailable."}}</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1000285776</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:37:00.325362+00:00</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:42 EDT</t>
+        </is>
+      </c>
+      <c r="R13" t="n">
+        <v>462</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:42:38.418569+00:00</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:16.035947+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1000285773</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>pricing_needed</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>assistant@jriley-law.com</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Nels Ramsay</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>5970 Plantation CT, Keystone Heights, FL 32656</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>{"total_amount": 0.0, "services": [], "pricing_reasoning": "The database lot size is 8.27 acres, which exceeds the 5.00-acre threshold requiring escalation for any service type. Although the aerial image analysis estimates approximately 2.5 acres (with LOW confidence due to dense canopy obscuring true parcel boundaries), the authoritative lot size on record is 8.27 acres and must govern pricing decisions. Additionally, the aerial analysis confidence is LOW, the legal description is missing, the county appraiser site was unreachable, and the aerial estimate diverges significantly from the DB value \u2014 all of which further support escalation rather than a standard price quote. This order must be reviewed by management before any price is issued.", "confidence": "LOW", "escalate_flag": true, "escalate_reason": "Database lot size of 8.27 acres exceeds the 5.00-acre escalation threshold for all service types. Aerial estimate of ~2.5 acres cannot override the recorded lot size, especially given LOW aerial confidence caused by dense pine canopy obscuring parcel boundaries. Additionally, the legal description is absent, the county appraiser site was unreachable, and there is a significant discrepancy between the DB size (8.27 ac) and aerial estimate (~2.5 ac). Management must verify true parcel size, confirm legal description, and issue a custom quote before fieldwork is scheduled.", "flags": ["LOT SIZE EXCEEDS 5.00 AC: DB value is 8.27 acres \u2014 mandatory escalation per pricing guidelines regardless of aerial estimate.", "AERIAL CONFIDENCE LOW: Dense tree canopy obstructs boundary visibility; aerial estimate of ~2.5 acres is unreliable and conflicts materially with DB lot size of 8.27 acres.", "LEGAL DESCRIPTION MISSING: No legal description provided; cannot confirm metes-and-bounds complexity or parcel identity without appraiser data.", "COUNTY APPRAISER SITE UNREACHABLE: Property details could not be independently verified at time of quote; parcel data should be confirmed before pricing.", "NEW CLIENT \u2014 ZERO ORDER HISTORY: Nels Ramsay / OLD_TITLE tier, 0 prior orders with NexGen; no negotiated rate on file. Default $400.00 base would apply once escalation is resolved.", "NO ELEVATION CERTIFICATE REQUESTED: Service is Land Survey Only; FEMA Zone X is non-mandatory flood zone \u2014 no EC line item warranted.", "MULTIPLE OUTBUILDINGS NOTED: Three visible structures plus a possible water tank/round structure on site; field crew should be briefed for potentially complex locate work once quote is approved."]}</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202606231443425880, "created_at": "2026-06-23T14:43:42", "customer_email": "assistant@jriley-law.com", "customer_id": 202606231443425984, "customer_name": "Nels Ramsay", "customer_type": "b2b", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12019C0375E\nZONE:X\nEFF: 03/17/2014", "invoiced": false, "order_id": 1000285773, "paid": false, "property_address": "5970 PLANTATION CT", "property_city": "KEYSTONE HEIGHTS", "property_county": "Clay County", "property_lat": "29.8642545", "property_lng": "-81.9060614", "property_state": "FLORIDA", "property_zip": "32656", "service_type": "Land Survey Only", "special_pricing": false, "status": "Quote", "status_code": 12, "updated_at": "2026-06-23T15:16:51"}, "ftf_customer": {"data": {"company_id": 202606231443425880, "company_name": "Nels Ramsay", "created_at": null, "custom_rate": null, "customer_id": 202606231443425984, "customer_type": "b2b", "email": "assistant@jriley-law.com", "first_name": "Nels Ramsay", "last_name": " ", "phone": "9044250040", "pricing_type": 0, "special_pricing": false}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": null, "source_url": "https://qpublic.schneidercorp.com/Application.aspx?AppID=830&amp;LayerID=15008&amp;PageTypeID=4&amp;PageID=6756&amp;Q=1806733921&amp;KeyValue=", "confidence": "LOW", "error": "Appraiser site unreachable (possible broken URL): https://qpublic.schneidercorp.com/Application.aspx?AppID=830&amp;LayerID=15008&amp;PageTypeID=4&amp;PageID=6756&amp;Q=1806733921&amp;KeyValue="}, "aerial_analysis": {"lot_shape": "irregular", "estimated_lot_size": "~2.5 acres", "main_structure_footprint_sqft": 1200, "visible_structures": ["main house or large shed (metal roof, center-right)", "smaller outbuilding or shed (red roof, left side)", "additional structure (white roof, upper right area)"], "driveway_count": 1, "pool_visible": false, "apparent_encroachments": "Structures appear to be set well within wooded boundary; no obvious encroachments visible, but dense tree canopy may obscure boundary features", "access_type": "unclear", "site_notes": "Property is heavily wooded with pine trees throughout; cleared area in center where structures are located. Multiple outbuildings present. Access path/driveway visible on right side leading to structures. Tree line may obscure true parcel boundaries. Elevation survey may need to account for varying terrain under dense canopy. A circular object (possibly a water tank or round structure) visible near center of clearing.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Nels Ramsay", "confidence": "HIGH"}, "client_email": {"value": "assistant@jriley-law.com", "confidence": "HIGH"}, "property_address": {"value": "5970 Plantation CT, Keystone Heights, FL 32656", "confidence": "HIGH"}, "property_county": {"value": "Clay County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated in order data; no elevation certificate requested."}, "special_requirements": {"value": "None noted", "confidence": "HIGH"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features available; county appraiser site unreachable and no matching emails found."}, "client_tier": {"value": "b2b", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Lot size unknown \u2014 county appraiser site unreachable", "Legal description unavailable \u2014 county appraiser site unreachable", "Structure square footage unknown", "Property features (pool, shed, outbuildings, fencing, driveways) unknown", "No matching emails found to supplement order details", "Fieldwork date not yet scheduled", "Invoice not yet generated \u2014 due amount is $0.00", "Estimate not yet sent to client"], "summary": "B2B Land Survey Only order for Nels Ramsay at 5970 Plantation CT, Keystone Heights, FL (Clay County), currently in Quote status with no fieldwork scheduled and property details unavailable due to unreachable county appraiser site."}}</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:37:26.143606+00:00</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:43:01.444821+00:00</t>
+        </is>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:43:01.453412+00:00</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:16.111852+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1000285707</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>details_missing</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>shailevitin@gmail.com</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Shai Levitin Shai Levitin</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>11876 PEBBLEWOOD DR</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:38:00.794030+00:00</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:38:00.803703+00:00</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:16.206140+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1000285630</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Land Survey and Elevation</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>kali@mondocklaw.com</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Kali Peley (Mondock Law PLLC)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>3731 5TH AVE NW, NAPLES, FL 34120</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>{"total_amount": 1549.0, "services": [{"name": "Land Survey (Boundary)", "description": "Base boundary survey at negotiated B2B rate for Mondock Law PLLC / Kali Peley \u2014 management-approved custom rate.", "amount": 450.0}, {"name": "Lot Size Complexity \u2014 2.01\u20135.00 ac", "description": "Property is 2.72 acres (confirmed by DB and aerial ~2.5 ac), falling in the 2.01\u20135.00 ac tier. Larger parcel requires extended boundary traversal and additional field time.", "amount": 550.0}, {"name": "Heavy Vegetation Upcharge", "description": "Aerial analysis confirms dense tree canopy across the full parcel. Boundary delineation is noted as difficult from aerial view; field crew will face obstructed sight lines, requiring additional time to locate corners and run traverse through heavy vegetation.", "amount": 112.0}, {"name": "Elevation Certificate (EC)", "description": "FEMA flood zone 12021C0410H \u2014 dual zones AH and X (eff. 05/16/2012). Zone AH is a special flood hazard area requiring a full Elevation Certificate. Zone is not VE (coastal), so no $50 VE surcharge applies. Standard EC rate applies.", "amount": 275.0}, {"name": "Pool Complexity Upcharge", "description": "Pool is confirmed visible in aerial imagery, located north of the main structure. Pool must be located and depicted on the survey sketch.", "amount": 62.0}, {"name": "Metes and Bounds Complexity", "description": "Legal description \u2014 'GOLDEN GATE EST UNIT 3 W 180FT OF TR 46' \u2014 describes a metes-and-bounds strip/fractional parcel (west 180 feet of Tract 46), requiring careful legal interpretation and precise distance/bearing control rather than a simple platted lot lookup.", "amount": 100.0}], "pricing_reasoning": "The management-approved negotiated rate of $450 is used as the base survey fee for Mondock Law PLLC. Complexity upcharges are applied for the 2.72-acre lot size ($550), confirmed heavy vegetation/dense canopy ($112), a visible pool ($62), and a metes-and-bounds fractional tract legal description ($100). The Elevation Certificate is priced at the standard $275 flat rate; the FEMA zones are AH and X \u2014 neither is VE, so no coastal surcharge is added. Multiple structures (possible ADU/guest house) and two driveways are noted as field considerations but do not independently carry their own line-item upcharges under current guidelines; they are absorbed within the existing complexity upcharges already applied.", "confidence": "MEDIUM", "escalate_flag": false, "escalate_reason": null, "flags": ["MULTIPLE_STRUCTURES: Aerial shows main house, detached garage/outbuilding, secondary structure (NW), pool, and shed (SE). Possible ADU or guest house. Field crew should confirm all structures are located and depicted; client or attorney should be advised if additional certifications per structure are needed.", "AERIAL_CONFIDENCE_LOW: Satellite analysis confidence is LOW due to dense canopy. Lot size estimated at ~2.5 ac aerially vs. 2.72 ac in DB \u2014 DB figure used for pricing tier. Field conditions may reveal additional complexity.", "DUAL_DRIVEWAY: Two separate driveways noted. Possible private road or shared easement along western boundary \u2014 field crew should verify easement status against OR 1955 PG 1031 and depict accordingly.", "TERRAIN_VARIATION: Dense canopy may obscure grade changes relevant to Elevation Certificate benchmarking. Surveyor should note if additional benchmarks or rod shots are needed for accurate FEMA BFE determination in Zone AH.", "ORDER_COUNT_ZERO: Mondock Law PLLC has 0 prior orders with NexGen. Client tier classified as OLD_TITLE (established title company). Negotiated rate confirmed per order notes \u2014 no further action needed, but relationship is new."]}</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202111241424361546, "created_at": "2026-06-18T21:02:18", "customer_email": "kali@mondocklaw.com", "customer_id": 202411051555164447, "customer_name": "Kali  Peley", "customer_type": "b2b", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12021C0410H\nZONE:AH\nZONE:X\nEFF: 05/16/2012", "invoiced": false, "order_id": 1000285630, "paid": false, "property_address": "3731 5TH AVE NW", "property_city": "NAPLES", "property_county": "COLLIER COUNTY", "property_lat": "26.2390296", "property_lng": "-81.6821317", "property_state": "FLORIDA", "property_zip": "34120", "service_type": "Land Survey and Elevation", "special_pricing": true, "status": "Quote", "status_code": 12, "updated_at": "2026-06-19T12:46:34"}, "ftf_customer": {"data": {"company_id": 202111241424361546, "company_name": "Mondock Law PLLC", "created_at": null, "custom_rate": 450.0, "customer_id": 202411051555164447, "customer_type": "b2b", "email": "kali@mondocklaw.com", "first_name": " Kali ", "last_name": "Peley", "phone": "2396732211", "pricing_type": 0, "special_pricing": true}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "Page unavailable at time of retrieval. Property address: 3731 5TH AVE NW, Collier County. Manual lookup may be required at https://www.collierappraiser.com", "source_url": "https://www.collierappraiser.com/search?address=3731%205TH%20AVE%20NW", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "irregular", "estimated_lot_size": "~2.5 acres", "main_structure_footprint_sqft": 3800, "visible_structures": ["main house", "detached garage or outbuilding", "secondary structure (northwest)", "pool", "shed or small outbuilding (southeast)"], "driveway_count": 2, "pool_visible": true, "apparent_encroachments": "null", "access_type": "street", "site_notes": "Property is heavily wooded with dense tree canopy making boundary delineation difficult from aerial view. Two separate driveways visible \u2014 one curving from south, one from northwest area. Multiple structures spread across parcel suggesting possible guest house or accessory dwelling units. Pool located north of main structure. Secondary smaller structure visible in southeast corner of property. Property appears to share a private road or easement along western boundary. Tree encroachment near structure setbacks warrants field verification. Elevation survey may need to account for varied terrain under dense canopy.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Kali Peley (Mondock Law PLLC)", "confidence": "HIGH"}, "client_email": {"value": "kali@mondocklaw.com", "confidence": "HIGH"}, "property_address": {"value": "3731 5TH AVE NW, NAPLES, FL 34120", "confidence": "HIGH"}, "property_county": {"value": "COLLIER COUNTY", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey", "Elevation Certificate"], "confidence": "HIGH", "notes": "Service type is listed as 'Land Survey and Elevation'; elevation_cert flag is false but service type explicitly includes elevation \u2014 likely a data entry inconsistency, needs human review."}, "special_requirements": {"value": "Special pricing applies; custom rate of $450.00 on file for this B2B client.", "confidence": "HIGH"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features, structures, pool, shed, or driveway details provided in any data source."}, "client_tier": {"value": "b2b", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Lot size is unknown \u2014 needed for accurate scoping and pricing", "Legal description is missing \u2014 required for survey deliverable", "Structure square footage not provided", "Property features unknown (pool, shed, fencing, driveways, etc.)", "elevation_cert flag is false but service type includes 'Elevation' \u2014 confirm if Elevation Certificate is actually required", "No supporting emails found to clarify scope or client intent", "Fieldwork date not yet scheduled", "Order has not been invoiced or paid \u2014 still in Quote status"], "summary": "B2B client Kali Peley of Mondock Law PLLC is requesting a Land Survey and Elevation Certificate for a residential property at 3731 5TH AVE NW, Naples, FL 34120 (Collier County), with special pricing at a $450 custom rate, currently in Quote status pending scope confirmation and scheduling."}}</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>1000285630</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:38:32.757925+00:00</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:43 EDT</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>1549</v>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:43:40.833289+00:00</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:16.284260+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1000285613</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>lisacline2000@yahoo.com</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Lisa Cline</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>VACANT LAND, WESLEY CHAPEL, FL 33543</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>{"total_amount": 612.0, "services": [{"name": "Land Survey Only", "description": "Boundary survey for vacant parcel in Wesley Chapel, Pasco County, FL. Base rate for individual client.", "amount": 475.0}, {"name": "Lot Size Complexity Upcharge (0.51\u20131.00 ac)", "description": "Property is recorded at 1.00 acre, falling within the 0.51\u20131.00 ac tier, warranting a field complexity upcharge for increased boundary work on a larger vacant parcel.", "amount": 137.0}], "pricing_reasoning": "This is a standard boundary survey (Land Survey Only) for an individual client, priced from the default base rate of $475.00. The lot is recorded at 1.00 acres, which falls within the 0.51\u20131.00 ac complexity tier, adding $137.00. No EC was requested, no pool, no waterfront canal, and the county is Pasco (not Monroe), so no additional upcharges apply. The FEMA Zone A designation does not trigger an EC line item since none was ordered.", "confidence": "LOW", "escalate_flag": true, "escalate_reason": "Multiple critical issues require human review before work is dispatched: (1) No street address or legal description has been provided \u2014 the parcel cannot be definitively identified or located without follow-up with the client. (2) No aerial imagery was available for this location, preventing any independent verification of lot shape, size, access, vegetation, or encroachments. (3) Three probable duplicate orders exist for the same coordinates and Folio/MLS number (Orders 1000095381, 1000277528, 1000278670) \u2014 this order should not proceed until those duplicates are reconciled. (4) FEMA Zone A with 'No Elevation Determined' may signal a high-risk flood area where an Elevation Certificate could be required by a lender or insurer; the client should be advised.", "flags": ["DUPLICATE_SUSPECTED: Order 1000095381 \u2014 32742 YASMINE LOOP, PASCO COUNTY \u2014 same coordinates (28.2107548, -82.2909146) \u2014 Land Survey Only", "DUPLICATE_SUSPECTED: Order 1000277528 \u2014 XXXX VACANT LAND, PASCO COUNTY \u2014 same coordinates and same Folio/MLS (15-26-20-0010-01500-0151) \u2014 Land Survey Only", "DUPLICATE_SUSPECTED: Order 1000278670 \u2014 XXXX VACANT LAND, PASCO COUNTY \u2014 same coordinates and same Folio/MLS (15-26-20-0010-01500-0151) \u2014 Land Survey Only", "MISSING_DATA: No street address provided \u2014 parcel identity unconfirmed", "MISSING_DATA: No legal description provided \u2014 cannot verify parcel boundaries or acreage", "NO_AERIAL_IMAGERY: Google Static Maps returned no imagery for this location \u2014 field visit or county GIS required before survey dispatch", "FEMA_ZONE_A_NO_BFE: Base Flood Elevation not determined \u2014 client may need EC for financing or insurance; recommend advisory outreach"]}</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202602131526258728, "created_at": "2026-06-18T19:01:33", "customer_email": "lisacline2000@yahoo.com", "customer_id": 202602131526258859, "customer_name": "Lisa Cline", "customer_type": "individual", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12101C0431F\nZONE: A\nNO ELEVATION DETERMINED\nEFFECTIVE: 09/26/2014", "invoiced": false, "order_id": 1000285613, "paid": false, "property_address": " VACANT LAND", "property_city": "WESLEY CHAPEL", "property_county": "PASCO COUNTY", "property_lat": "28.2107548", "property_lng": "-82.2909146", "property_state": "FL", "property_zip": "33543", "service_type": "Land Survey Only", "special_pricing": false, "status": "Quote", "status_code": 12, "updated_at": "2026-06-18T19:30:32"}, "ftf_customer": {"data": {"company_id": 202602131526258728, "company_name": "Lisa Cline", "created_at": null, "custom_rate": null, "customer_id": 202602131526258859, "customer_type": "individual", "email": "lisacline2000@yahoo.com", "first_name": "Lisa Cline", "last_name": " ", "phone": "920-226-0939", "pricing_type": 0, "special_pricing": false}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "No specific property data found. The page returned is the Pasco County Records Search landing/home page, not a specific parcel detail page. The address 'VACANT LAND' did not resolve to a specific parcel record.", "source_url": "http://search.pascopa.com/?address=%20VACANT%20LAND", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "other", "estimated_lot_size": null, "main_structure_footprint_sqft": null, "visible_structures": [], "driveway_count": null, "pool_visible": false, "apparent_encroachments": null, "access_type": "unclear", "site_notes": "No aerial imagery available for this location. The map tile returned a 'Sorry, we have no imagery here' error via Google Static Maps API. A field visit or alternative imagery source (county GIS, NAIP, nearmap) is required to complete the aerial analysis for this vacant land parcel.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Lisa Cline", "confidence": "HIGH"}, "client_email": {"value": "lisacline2000@yahoo.com", "confidence": "HIGH"}, "property_address": {"value": "VACANT LAND, WESLEY CHAPEL, FL 33543", "confidence": "MEDIUM"}, "property_county": {"value": "PASCO COUNTY", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey Only"], "confidence": "HIGH", "notes": "Service type explicitly stated as 'Land Survey Only'; no elevation certificate requested"}, "special_requirements": {"value": "Property is in Flood Zone A (FEMA panel 12101C0431F, effective 09/26/2014) with no base flood elevation determined. Vacant land with no structure.", "confidence": "MEDIUM"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "HIGH"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "Vacant land only; no structures, pool, shed, or other features known \u2014 field verification required"}, "client_tier": {"value": "residential", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["No street address provided \u2014 only 'VACANT LAND'; parcel ID or legal description needed to locate property", "Lot size unknown", "Legal description not provided", "No parcel number or folio ID supplied", "No emails on file to cross-reference order details", "Flood zone is Zone A with no BFE determined \u2014 elevation certificate not ordered but may be relevant depending on lender requirements", "Urgency/deadline not stated"], "summary": "Individual client Lisa Cline has requested a Land Survey Only for a vacant parcel in Wesley Chapel, Pasco County, FL (Flood Zone A), but no street address or legal description has been provided, requiring follow-up to identify the exact parcel."}}</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>1000285613</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:39:05.500395+00:00</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:44 EDT</t>
+        </is>
+      </c>
+      <c r="R17" t="n">
+        <v>612</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:44:09.246536+00:00</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:16.348396+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1000285607</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Land Survey and Elevation</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>daniel.hysa@compass.com</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Daniel Hysa</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>6065 Pine Tree Dr, Miami Beach, FL 33140</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>{"total_amount": 899.0, "services": [{"name": "Boundary/Land Survey", "description": "Base residential boundary survey for individual client at 6065 Pine Tree Dr, Miami-Dade County. Irregular waterfront lot ~0.24\u20130.25 acres on canal with private dock.", "amount": 475.0}, {"name": "Elevation Certificate", "description": "FEMA Elevation Certificate for FEMA Flood Zone AE (panel 12086C0328L, eff. 09/11/2009). Standard EC rate; Zone AE does not trigger the VE coastal surcharge.", "amount": 275.0}, {"name": "Waterfront Canal Complexity Upcharge", "description": "Property is a canal-front lot with a private dock extending into the waterway. Aerial confirms direct water access at rear. Riparian boundary, mean high water line determination, and dock structure coordination add measurable field complexity.", "amount": 87.0}, {"name": "Pool Complexity Upcharge", "description": "Swimming pool confirmed visible in aerial imagery. Pool must be located and tied into the boundary survey for a complete depiction of improvements.", "amount": 62.0}], "pricing_reasoning": "This is a combined boundary survey plus Elevation Certificate order for a residential waterfront lot in Miami-Dade County (Zone AE). The base individual client rate of $475.00 applies for the boundary survey, plus the flat $275.00 EC fee. Two complexity upcharges are supported by aerial evidence: the canal-front dock situation (+$87.00) and the in-ground swimming pool (+$100 cap, guideline $62.00). The lot at ~0.24 acres falls within the base tier (\u22640.30 ac), so no acreage upcharge applies. Zone is AE, not VE, so no coastal EC surcharge. Heavy vegetation was noted as a possible factor at boundary edges but confidence is LOW on that observation, so it is not applied; the waterfront upcharge already captures the access/boundary difficulty at the rear of the lot.", "confidence": "MEDIUM", "escalate_flag": false, "escalate_reason": null, "flags": ["AERIAL_CONFIDENCE_LOW: Google satellite analysis returned LOW confidence \u2014 field crew should verify pool dimensions, dock extent, and boundary vegetation conditions on-site before commencing work.", "RIPARIAN_RIGHTS_NOTE: Aerial shows dock extending into canal; riparian boundary and mean high water line determination may require additional scope. If client or title requires MHW line delineation as a separate deliverable, escalate for supplemental pricing.", "NO_LEGAL_DESCRIPTION: Legal description field is blank. Crew/office should obtain the recorded plat or legal description before scheduling fieldwork to confirm lot geometry and platted easements.", "NEW_CLIENT: Daniel Hysa has 0 prior orders with NexGen \u2014 no negotiated rate history; default individual pricing applied."]}</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202606181832520052, "created_at": "2026-06-18T18:32:52", "customer_email": "daniel.hysa@compass.com", "customer_id": 202606181832520160, "customer_name": "Daniel Hysa", "customer_type": "individual", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": "12086C0328L\nZONE:AE\nEFF: 09/11/2009", "invoiced": false, "order_id": 1000285607, "paid": false, "property_address": "6065 PINE TREE DR", "property_city": "MIAMI BEACH", "property_county": "MIAMI-DADE COUNTY", "property_lat": "25.842089", "property_lng": "-80.124586", "property_state": "FLORIDA", "property_zip": "33140", "service_type": "Land Survey and Elevation", "special_pricing": false, "status": "Quote", "status_code": 12, "updated_at": "2026-06-18T18:55:30"}, "ftf_customer": {"data": {"company_id": 202606181832520052, "company_name": "Daniel Hysa", "created_at": null, "custom_rate": null, "customer_id": 202606181832520160, "customer_type": "individual", "email": "daniel.hysa@compass.com", "first_name": "Daniel Hysa", "last_name": " ", "phone": "425.218.9349", "pricing_type": 0, "special_pricing": false}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "No property data was returned from the Miami-Dade County search page. The page only shows a search interface with no results visible in the provided text. A direct lookup via the Miami-Dade County Property Appraiser (https://www.miamidade.gov/Apps/PA/propertysearch/) using the folio number or address may be required to retrieve parcel details for 6065 Pine Tree Dr.", "source_url": "https://www.miamidade.gov/search?address=6065%20PINE%20TREE%20DR", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "irregular", "estimated_lot_size": "~0.25 acres", "main_structure_footprint_sqft": 2800, "visible_structures": ["main house", "swimming pool", "private dock/boat dock", "paved driveway", "landscaping/garden structures"], "driveway_count": 1, "pool_visible": true, "apparent_encroachments": "Dock structure extends into waterway; vegetation along property boundaries may obscure exact boundary lines", "access_type": "street", "site_notes": "Property appears to be a waterfront lot along a canal in what appears to be Miami Beach/Bay Harbor Islands area. Rear of property has direct water access with a private dock. Elevation survey recommended given proximity to water and potential flood zone designation. Riparian rights and dock permit verification advised. Street frontage on Pine Tree Drive (western side). Lot appears wider at water frontage than street frontage, contributing to irregular shape. Adjacent properties have similar dock structures. Mean high water line determination may be necessary for boundary survey.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Daniel Hysa", "confidence": "HIGH"}, "client_email": {"value": "daniel.hysa@compass.com", "confidence": "HIGH"}, "property_address": {"value": "6065 Pine Tree Dr, Miami Beach, FL 33140", "confidence": "HIGH"}, "property_county": {"value": "Miami-Dade County", "confidence": "HIGH"}, "services_requested": {"value": ["Boundary Survey", "Elevation Certificate"], "confidence": "MEDIUM", "notes": "Service type listed as 'Land Survey and Elevation' \u2014 interpreted as boundary/land survey plus elevation certificate, though elevation_cert flag is set to false; confirm which specific survey products are required"}, "special_requirements": {"value": null, "confidence": "LOW"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features available; no emails or attachments found. Pool, dock, seawall, or other waterfront features common in Miami Beach \u2014 field inspection or aerial review needed."}, "client_tier": {"value": "residential", "confidence": "MEDIUM"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "ftf_only", "gaps": ["Elevation certificate flag is false but service type includes 'Elevation' \u2014 confirm whether EC is required", "Lot size unknown", "Legal description not provided", "Structure square footage unknown", "Property features (pool, dock, seawall, fence, outbuildings) not documented", "Special requirements or client notes absent", "No matching emails found \u2014 no additional context from client communication", "Flood zone AE confirmed (12086C0328L, eff. 09/11/2009) \u2014 base flood elevation data should be verified at time of fieldwork", "Fieldwork and delivery dates not yet scheduled", "Invoice not yet created and no pricing established"], "summary": "Residential land survey and elevation order for Daniel Hysa at 6065 Pine Tree Dr, Miami Beach (Flood Zone AE), currently in Quote status with no fieldwork scheduled, pricing, or supporting documentation on file."}}</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>1000285607</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:39:38.393976+00:00</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:44 EDT</t>
+        </is>
+      </c>
+      <c r="R18" t="n">
+        <v>899</v>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:44:38.599371+00:00</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:16.429988+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1000285579</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>dina@professionaltitleirc.com</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Dina Robinson</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>CO RD 512, Indian River County, FL</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>{"total_amount": 575.0, "services": [{"name": "Land Survey (Boundary)", "description": "Negotiated base survey rate for Professional Title of Indian River, Inc. (OLD_TITLE client tier, agreed management rate).", "amount": 300.0}, {"name": "Lot Size Complexity Upcharge (1.01\u20132.00 ac per DB)", "description": "Database lot size is listed as 1.26 acres, falling in the 1.01\u20132.00 ac tier. Aerial analysis estimates ~0.25 ac, but confidence is LOW due to mature tree coverage, rural intersection ambiguity, and incomplete address data. Per pricing guidelines, the DB lot size governs; upcharge applied at the 1.01\u20132.00 ac tier rate.", "amount": 275.0}], "pricing_reasoning": "The client holds a negotiated base rate of $300.00 as an established title company (OLD_TITLE tier). The database lot size of 1.26 acres triggers the 1.01\u20132.00 ac complexity upcharge of $275.00; aerial confidence is LOW due to mature canopy cover, an incomplete address, and an unreachable county appraiser site, so the DB figure is used as the authoritative lot size per standard protocol. No pool, waterfront, metes-and-bounds, or Monroe County factors are present; the FEMA zone includes Zone A but no Elevation Certificate was ordered, so no EC line item applies.", "confidence": "LOW", "escalate_flag": true, "escalate_reason": "Multiple data quality concerns warrant management review before invoice is finalized: (1) The aerial image confidence is LOW \u2014 mature tree coverage obscures boundaries and the ~0.25 ac aerial estimate conflicts sharply with the 1.26 ac DB lot size, which directly affects which complexity upcharge tier applies and therefore the invoice total. (2) The property address is incomplete ('CO RD 512' only) and the Indian River County Property Appraiser site was unreachable, leaving the legal description blank \u2014 field crew cannot be dispatched without a verified legal description or parcel ID. (3) A possible duplicate order (1000285342) exists for the same location and service type \u2014 management should confirm whether this is a re-order, a different parcel at the same intersection, or a billing duplicate before proceeding.", "flags": ["POSSIBLE_DUPLICATE: Order 1000285342 \u2014 same location (CO RD 512, Indian River County), same service (Land Survey Only) \u2014 coordinate with management to confirm this is not a duplicate billing or re-order before proceeding.", "INCOMPLETE_ADDRESS: Property address is 'CO RD 512' only \u2014 no parcel number, no legal description, and county appraiser site was unreachable. Legal description must be obtained before field work can be scheduled.", "LOT_SIZE_CONFLICT: DB lot size (1.26 ac) vs. aerial estimate (~0.25 ac) are significantly divergent. Aerial confidence is LOW due to canopy obscuring boundaries at a rural multi-lot intersection. DB size used for pricing per standard protocol, but field verification is critical.", "COMMERCIAL_FLAG: Order is flagged commercial \u2014 if the property is confirmed as commercial rather than residential, pricing may need re-evaluation by management.", "MULTI_CERT: Four certifications listed (k91 training &amp; consulting llc, First National Bank Coastal Community, Professional Title of the Treasure Coast, Commonwealth Land Title Insurance) \u2014 confirm whether additional certification copies or split invoicing is required."]}</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"order_id": "1000285579", "customer_email": "dina@professionaltitleirc.com", "service_type": "Land Survey Only", "county": "Indian River County", "property_address": "CO RD 512", "customer_name": "Dina Robinson"}, "ftf_customer": {}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": null, "source_url": "https://qpublic.schneidercorp.com/Application.aspx?AppID=1109&amp;LayerID=27655&amp;PageTypeID=4&amp;PageID=11279&amp;Q=1447726964&amp;KeyValue=", "confidence": "LOW", "error": "Appraiser site unreachable (possible broken URL): https://qpublic.schneidercorp.com/Application.aspx?AppID=1109&amp;LayerID=27655&amp;PageTypeID=4&amp;PageID=11279&amp;Q=1447726964&amp;KeyValue="}, "aerial_analysis": {"lot_shape": "rectangular", "estimated_lot_size": "~0.25 acres", "main_structure_footprint_sqft": 1200, "visible_structures": ["main house", "detached garage", "shed"], "driveway_count": 1, "pool_visible": false, "apparent_encroachments": null, "access_type": "street", "site_notes": "Property appears to be located at a rural intersection with County Road 512. Multiple residential lots visible at four-way intersection. Mature tree coverage on most lots may obscure boundary markers and structure details. Gravel/dirt road surfaces suggest rural setting. Several outbuildings visible across the intersection area. Lot boundaries are estimated based on visual separation between properties; field verification recommended.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Dina Robinson", "confidence": "HIGH"}, "client_email": {"value": "dina@professionaltitleirc.com", "confidence": "HIGH"}, "property_address": {"value": "CO RD 512, Indian River County, FL", "confidence": "MEDIUM"}, "property_county": {"value": "Indian River County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey"], "confidence": "HIGH", "notes": "Service type listed as 'Land Survey Only' \u2014 specific survey type (boundary, ALTA, topo, etc.) not specified"}, "special_requirements": {"value": null, "confidence": "LOW"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property appraiser data available and no emails or attachments to reference; features unknown"}, "client_tier": {"value": "b2b", "confidence": "MEDIUM"}, "urgency": {"value": "unknown", "confidence": "LOW"}, "source_of_truth": "ftf_only", "gaps": ["Full street address \u2014 'CO RD 512' lacks a street number or parcel-level specificity", "Parcel ID / folio number needed to look up property appraiser records", "Legal description not available (appraiser site unreachable)", "Lot size / acreage unknown", "Specific survey type not defined (boundary, ALTA, topographic, etc.)", "Property features unknown (structures, pool, fence, encroachments, etc.)", "Structure square footage unknown", "Special requirements or notes not provided", "Urgency / turnaround expectation not stated", "Client tier confirmation \u2014 email domain suggests title company (b2b) but not confirmed"], "summary": "Dina Robinson of Professional Title IRC is requesting a land survey on a property located on CO RD 512 in Indian River County, with significant data gaps due to an incomplete address and an unreachable property appraiser site."}}</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>1000285579</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:40:02.969986+00:00</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:45 EDT</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>575</v>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:45:11.617878+00:00</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:16.502296+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1000285516</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>pricing_needed</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Land Survey Only</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>rfrankel@frankel-realty.com</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Frankel Construction</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>12477 Seminole Blvd</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>{"total_amount": 0.0, "services": [], "pricing_reasoning": "This order cannot be safely priced without escalation. Three prior orders exist for the identical property (same folio, same address, same coordinates), including a prior Land Survey Only (1000280518) and a Land Survey + Elevation (1000276040), creating a high likelihood of duplication. Additionally, the aerial analysis flags the lot at approximately 2.5 acres while the database shows 1.31 acres \u2014 a significant discrepancy that materially affects which lot-size upcharge tier applies. The order notes explicitly state that the survey type and property details need clarification before proceeding, and the aerial reveals substantial complexity (waterfront riparian boundary, dock, multiple structures, heavy tropical vegetation) that warrants management review before quoting.", "confidence": "LOW", "escalate_flag": true, "escalate_reason": "Multiple escalation triggers present: (1) Three confirmed duplicate orders at the same folio/location (1000276040, 1000280518, 1000284871) \u2014 status and scope of prior orders must be resolved before pricing a new one; (2) Lot size conflict \u2014 database says 1.31 ac but aerial estimate is ~2.5 ac, a difference that shifts the complexity upcharge from +$275 to +$550 and must be verified against the plat or county records before pricing; (3) Order notes explicitly flag that survey type and property details need clarification from Frankel Construction; (4) Aerial analysis confidence is LOW and identifies a riparian/waterway western boundary requiring mean high water line determination \u2014 this is a non-standard boundary condition that may require a separate scope discussion; (5) Secondary structures, potential setback issues, and dock/boat slip add scope ambiguity that management should confirm with the client before a price is issued.", "flags": ["DUPLICATE_RISK: Order 1000276040 \u2014 same address 12477 SEMINOLE BLVD, Palm Beach County \u2014 service: Land Survey and Elevation \u2014 same folio 00434133090000140. Verify if that order was completed, cancelled, or is still active.", "DUPLICATE_RISK: Order 1000280518 \u2014 same address 12477 SEMINOLE BLVD, Palm Beach County \u2014 service: Land Survey Only \u2014 same folio 00434133090000140. This is the same service type as the current order; confirm this is not a re-submission.", "DUPLICATE_RISK: Order 1000284871 \u2014 same address 12477 SEMINOLE BLVD, Palm Beach County \u2014 service: Quote \u2014 same folio 00434133090000140. A prior quote request exists; check whether a price was already issued.", "LOT_SIZE_CONFLICT: Database reports 1.31 acres; aerial analysis estimates ~2.5 acres. Must confirm against recorded plat (Plat Book 30, Page 35, Palm Beach County) before applying lot-size upcharge tier.", "SCOPE_UNCLEAR: Order notes state survey type and property details need clarification with Frankel Construction before proceeding.", "RIPARIAN_BOUNDARY: Canal/waterway along western property edge likely requires mean high water line or riparian boundary determination \u2014 non-standard field work that may require a scope and price adjustment.", "FEMA_AE_ZONE: Property is in Zone AE at 6 ft BFE (panel 12099C0381G, effective 12/20/2024). Elevation Certificate may be warranted given waterfront proximity; confirm with client whether EC is needed in addition to boundary survey.", "CLIENT_NEW: Frankel Construction has 0 prior orders with NexGen despite OLD_TITLE tier classification. Confirmed negotiated base rate of $475.00 is on file per management."]}</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"order_id": "1000285516", "customer_email": "rfrankel@frankel-realty.com", "service_type": "Land Survey Only", "county": "Palm Beach County", "property_address": "12477 SEMINOLE BLVD", "customer_name": "Frankel Construction"}, "ftf_customer": {}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": "No property-specific data was returned for 12477 SEMINOLE BLVD, Palm Beach County. The page text contains only general website content, navigation elements, and county statistics. The property detail page did not render or return usable parcel data.", "source_url": "https://pbcpao.gov/?address=12477%20SEMINOLE%20BLVD", "error": null, "confidence": "LOW"}, "aerial_analysis": {"lot_shape": "irregular", "estimated_lot_size": "~2.5 acres", "main_structure_footprint_sqft": 6500, "visible_structures": ["main house", "secondary/guest structure", "swimming pool", "multiple outbuildings or garages", "circular driveway feature", "dock or boat slip"], "driveway_count": 2, "pool_visible": true, "apparent_encroachments": "Vegetation and landscaping appear to extend heavily toward property boundaries; waterway along western edge may present riparian boundary considerations", "access_type": "street", "site_notes": "Property borders a canal/waterway on the western side, which will require riparian or mean high water line determination for boundary survey. Dense tropical landscaping throughout makes ground-level boundary verification important. A road or easement corridor runs along the northern edge. Multiple structures on parcel suggest potential need for improvement location certificate. Elevation survey may be warranted given proximity to water. Secondary structures in southern portion of lot may require setback verification. Golf course or recreational green space visible to north across road.", "confidence": "LOW"}, "packet": {"client_name": {"value": "Frankel Construction", "confidence": "HIGH"}, "client_email": {"value": "rfrankel@frankel-realty.com", "confidence": "HIGH"}, "property_address": {"value": "12477 Seminole Blvd", "confidence": "HIGH"}, "property_county": {"value": "Palm Beach County", "confidence": "HIGH"}, "services_requested": {"value": ["Land Survey"], "confidence": "HIGH", "notes": "Service type listed as 'Land Survey Only' \u2014 specific survey type (boundary, elevation, topographic, etc.) not specified"}, "special_requirements": {"value": null, "confidence": "LOW"}, "lot_size": {"value": null, "confidence": "LOW"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": null, "confidence": "LOW"}, "property_features": {"value": {}, "confidence": "LOW", "notes": "No property features available \u2014 no emails, attachments, or appraiser data provided"}, "client_tier": {"value": "b2b", "confidence": "MEDIUM"}, "urgency": {"value": "unknown", "confidence": "LOW"}, "source_of_truth": "ftf_only", "gaps": ["Specific survey type not clarified (boundary, elevation certificate, topographic, ALTA, etc.)", "Lot size unknown", "Legal description not provided", "Structure square footage unknown", "Property features not available (pool, shed, fences, driveways, etc.)", "Special requirements or client notes missing", "Urgency/turnaround expectations not stated", "No supporting emails or documents to cross-reference", "State not explicitly confirmed (assumed Florida based on Palm Beach County context)"], "summary": "B2B land survey order for Frankel Construction at 12477 Seminole Blvd in Palm Beach County, FL \u2014 specific survey type and property details need clarification before proceeding."}}</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:41:04.934964+00:00</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:45:39.449320+00:00</t>
+        </is>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:45:39.459440+00:00</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:16.573378+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1000285511</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>invoice_draft_posted</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>mjwygant@closewithbell.com</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>M Wygant</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>12955 SW Kanne Highway, Indiantown, FL 34956</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>{"total_amount": 1286.0, "services": [{"name": "Boundary Survey \u2013 Base Rate (Individual)", "description": "Standard boundary survey base rate for individual residential client M Wygant. No negotiated rate on file; default individual rate applied.", "amount": 475.0}, {"name": "Lot Size Upcharge \u2013 1.01 to 2.00 Acres", "description": "Property is approximately 1.5 acres (irregular lot), confirmed by aerial analysis. Applies the 1.01\u20132.00 ac tier upcharge for additional field time and boundary linework on a larger parcel.", "amount": 275.0}, {"name": "Waterfront / Dock Complexity Upcharge", "description": "Property has direct waterfront access with a private dock extending into a waterway. Waterfront boundary delineation and dock encroachment analysis add measurable field complexity. Standard waterfront canal upcharge applied.", "amount": 87.0}, {"name": "Pool Upcharge", "description": "Swimming pool is confirmed visible in aerial imagery adjacent to the main house. Pool must be located and shown on the survey.", "amount": 62.0}, {"name": "Heavy Vegetation / Tree Canopy Upcharge", "description": "Aerial imagery shows significant tree coverage across the lot, particularly near the waterfront boundary, which may obscure monuments and boundary markers and require additional field effort to clear sight lines.", "amount": 112.0}, {"name": "Elevation Certificate (EC) \u2013 Recommended", "description": "Property is waterfront with proximity to open water. FEMA flood zone not confirmed in order data, but waterfront location in Indiantown, Martin County strongly warrants an EC. Quoted as a recommended add-on at standard flat rate. No Zone VE surcharge applied as flood zone is unconfirmed.", "amount": 275.0}], "pricing_reasoning": "Base rate of $475.00 is applied as the default individual client rate with no negotiated pricing on file. Complexity upcharges are supported by aerial evidence: the 1.5-acre irregular lot triggers the 1.01\u20132.00 ac tier (+$275), the confirmed dock on a waterway triggers the waterfront upcharge (+$87), the visible pool triggers the pool upcharge (+$62), and heavy tree canopy near the waterfront boundary triggers the vegetation upcharge (+$112). An Elevation Certificate is quoted separately at $275 as a strongly recommended add-on given the open-water waterfront exposure, though it remains optional pending client confirmation. No FEMA zone was provided so no VE surcharge is applied; if the zone confirms as VE, add $50 to the EC line item.", "confidence": "MEDIUM", "escalate_flag": true, "escalate_reason": "Several scoping gaps warrant management review before finalizing: (1) No specific survey service has been selected by the client \u2014 boundary survey and EC are assumed but not confirmed. (2) No legal description or FEMA flood zone is on file, which affects both scope and EC pricing. (3) The metes-and-bounds upcharge (+$100) was intentionally withheld because the legal description is absent and cannot be confirmed; management should verify platted vs. metes-and-bounds upon retrieving the legal description and apply accordingly. (4) Multiple outbuildings (detached garage, small shed) are present and should be confirmed as in-scope for location. (5) The dock encroachment into the waterway may require additional boundary or mean high water line delineation beyond a standard survey. Management should confirm full scope with client before issuing a binding quote.", "flags": ["No survey service type selected by client \u2014 boundary survey assumed pending confirmation.", "FEMA flood zone unknown \u2014 EC priced at $275.00 flat; add $50.00 if Zone VE is confirmed.", "Legal description not provided \u2014 metes-and-bounds upcharge ($100.00) NOT applied; must be verified and added if applicable.", "Dock extends into waterway \u2014 may require mean high water line or riparian boundary delineation beyond standard scope.", "Multiple outbuildings present (detached garage, small shed) \u2014 confirm all structures are in scope for location.", "First-time client (0 prior orders) \u2014 no pricing history available for reference.", "Elevation Certificate listed as recommended add-on, not confirmed by client."]}</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>{"ftf_order": {"company_id": 202606171519217188, "created_at": "2026-06-17T15:19:21", "customer_email": "mjwygant@closewithbell.com", "customer_id": 202606171519217292, "customer_name": "M Wygant", "customer_type": "individual", "delivered_at": null, "due_amount": 0.0, "elevation_cert": false, "estimate_sent": false, "fieldwork_at": null, "flood_zone": null, "invoiced": false, "order_id": 1000285511, "paid": false, "property_address": "12955 SW KANNE HIGHWAY", "property_city": "INDIANTOWN", "property_county": "Martin County", "property_lat": "27.0216288", "property_lng": "-80.4316442", "property_state": "FLORIDA", "property_zip": "34956", "service_type": "Quote", "special_pricing": false, "status": "Quote", "status_code": 12, "updated_at": "2026-06-17T15:19:22"}, "ftf_customer": {"data": {"company_id": 202606171519217188, "company_name": "M Wygant", "created_at": null, "custom_rate": null, "customer_id": 202606171519217292, "customer_type": "individual", "email": "mjwygant@closewithbell.com", "first_name": "M Wygant", "last_name": " ", "phone": "561-385-0621", "pricing_type": 0, "special_pricing": false}, "success": true}, "emails_found": 0, "email_snippets": [], "appraiser_data": {"legal_description": null, "lot_size": null, "structure_sqft": null, "parcel_id": null, "year_built": null, "notes": null, "source_url": "https://www.pa.martin.fl.us/app/search/view/", "confidence": "LOW", "error": "Appraiser site unreachable (possible broken URL): https://www.pa.martin.fl.us/app/search/view/"}, "aerial_analysis": {"lot_shape": "irregular", "estimated_lot_size": "~1.5 acres", "main_structure_footprint_sqft": 3200, "visible_structures": ["main house", "detached garage or outbuilding", "swimming pool", "dock/boat dock", "small shed or storage structure"], "driveway_count": 1, "pool_visible": true, "apparent_encroachments": "Dock structure extends into waterway; vegetation and tree canopy may obscure boundary lines near water's edge", "access_type": "street", "site_notes": "Property is waterfront with direct access to a lake or river via a private dock. Roadway (SW Kanne Highway) runs diagonally along the southern boundary. The lot appears to have significant tree coverage which may obscure boundary markers. Waterfront boundary delineation will require additional survey work. Elevation survey recommended given proximity to open water. A secondary outbuilding is visible to the northeast of the main structure. The pool is located adjacent to the main house on the west side.", "confidence": "MEDIUM"}, "packet": {"client_name": {"value": "M Wygant", "confidence": "HIGH"}, "client_email": {"value": "mjwygant@closewithbell.com", "confidence": "HIGH"}, "property_address": {"value": "12955 SW Kanne Highway, Indiantown, FL 34956", "confidence": "HIGH"}, "property_county": {"value": "Martin County", "confidence": "HIGH"}, "services_requested": {"value": ["Boundary Survey", "Elevation Certificate"], "confidence": "MEDIUM", "notes": "Service type is listed only as 'Quote' with no specific survey type selected. Boundary survey inferred due to waterfront complexity, irregular lot, and encroachments. Elevation certificate strongly recommended given waterfront proximity to open water, but elevation_cert flag is false \u2014 needs confirmation from client."}, "special_requirements": {"value": "Waterfront boundary delineation required; dock extends into waterway; significant tree canopy may obscure boundary markers near water's edge; elevation survey recommended due to open water proximity", "confidence": "MEDIUM"}, "lot_size": {"value": "~1.5 acres", "confidence": "MEDIUM"}, "legal_description": {"value": null, "confidence": "LOW"}, "structure_sqft": {"value": 3200, "confidence": "MEDIUM"}, "property_features": {"value": {"pool": true, "dock": true, "detached_garage_or_outbuilding": true, "small_shed_or_storage": true, "driveways": 1, "waterfront": true, "tree_coverage": "significant", "road_along_boundary": "SW Kanne Highway runs diagonally along southern boundary"}, "confidence": "MEDIUM", "notes": "All features derived from aerial image analysis at medium confidence. County appraiser data unavailable to cross-reference. Pool flag in order data is false but aerial clearly shows pool \u2014 discrepancy needs review."}, "client_tier": {"value": "residential", "confidence": "HIGH"}, "urgency": {"value": "normal", "confidence": "MEDIUM"}, "source_of_truth": "mixed", "gaps": ["Specific survey service type not selected \u2014 order is in 'Quote' status only", "Legal description unavailable \u2014 county appraiser site unreachable", "Parcel ID / folio number unknown", "Elevation certificate intent unclear \u2014 flag is false but waterfront location warrants confirmation", "Pool feature discrepancy \u2014 aerial shows pool but order data has elevation_cert and pool-related flags as false", "No prior survey or deed provided for reference", "Fieldwork date not scheduled", "No matching emails found to clarify scope or client intent", "Flood zone classification unknown \u2014 needs FEMA FIRM panel lookup", "Waterfront boundary type unclear \u2014 lake vs. river vs. canal needs confirmation for scoping"], "summary": "Individual residential client M Wygant is requesting a quote for an irregular ~1.5-acre waterfront property in Indiantown, Martin County, FL, featuring a main house, pool, dock, and outbuildings, with no specific survey service selected and significant scoping details still needed."}}</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>1000285511</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:41:39.893315+00:00</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:46 EDT</t>
+        </is>
+      </c>
+      <c r="R21" t="n">
+        <v>1286</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:46:18.589730+00:00</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:33:16.659763+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>